<commit_message>
Atualização automática: vencimentos_tmot (15/09/2026 08:55)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (15/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (15/09/2026 14:02)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (16/09/2026 12:25)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (16/09/2026 12:40)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (17/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,16 +1019,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1044,7 +1036,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1052,30 +1044,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1375,37 +1349,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1434,7 +1408,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1466,7 +1440,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1498,7 +1472,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1530,7 +1504,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1562,7 +1536,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1594,7 +1568,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1626,7 +1600,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1658,7 +1632,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1690,7 +1664,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1722,7 +1696,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1754,7 +1728,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1786,7 +1760,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1818,7 +1792,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1850,7 +1824,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1882,7 +1856,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1914,7 +1888,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1946,7 +1920,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1978,7 +1952,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -2010,7 +1984,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2042,7 +2016,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2074,7 +2048,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2106,7 +2080,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2138,7 +2112,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2170,7 +2144,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2202,7 +2176,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2234,7 +2208,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2266,7 +2240,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2298,7 +2272,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2330,7 +2304,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2362,7 +2336,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2394,7 +2368,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2426,7 +2400,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2458,7 +2432,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2490,7 +2464,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2522,7 +2496,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2554,7 +2528,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2586,7 +2560,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2618,7 +2592,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2650,7 +2624,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2682,7 +2656,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2714,7 +2688,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2746,7 +2720,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2778,7 +2752,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2810,7 +2784,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2842,7 +2816,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2874,7 +2848,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2906,7 +2880,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2938,7 +2912,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2970,7 +2944,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -3002,7 +2976,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3034,7 +3008,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3066,7 +3040,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3098,7 +3072,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3130,7 +3104,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3162,7 +3136,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3194,7 +3168,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3226,7 +3200,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3258,7 +3232,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3290,7 +3264,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3322,7 +3296,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3354,7 +3328,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3386,7 +3360,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3418,7 +3392,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3450,7 +3424,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3482,7 +3456,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3514,7 +3488,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3546,7 +3520,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3578,7 +3552,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3610,7 +3584,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3642,7 +3616,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3674,7 +3648,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3706,7 +3680,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3738,7 +3712,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3770,7 +3744,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3802,7 +3776,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3834,7 +3808,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3866,7 +3840,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3901,7 +3875,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3936,7 +3910,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3971,7 +3945,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -4006,7 +3980,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4041,7 +4015,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4076,7 +4050,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4111,7 +4085,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4146,7 +4120,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4181,7 +4155,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4216,7 +4190,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4251,7 +4225,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4286,7 +4260,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4321,7 +4295,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4356,7 +4330,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4391,7 +4365,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4426,7 +4400,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4461,7 +4435,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4496,7 +4470,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4531,7 +4505,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4566,7 +4540,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4601,7 +4575,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4636,7 +4610,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4671,7 +4645,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4706,7 +4680,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4741,7 +4715,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4776,7 +4750,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4811,7 +4785,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4846,7 +4820,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4881,7 +4855,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4916,7 +4890,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4951,7 +4925,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4986,7 +4960,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -5021,7 +4995,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5056,7 +5030,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5091,7 +5065,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5126,7 +5100,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5161,7 +5135,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5196,7 +5170,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5231,7 +5205,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5266,7 +5240,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5301,7 +5275,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5336,7 +5310,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5371,7 +5345,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5406,7 +5380,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5441,7 +5415,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5476,7 +5450,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5511,7 +5485,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5546,7 +5520,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5581,7 +5555,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5616,7 +5590,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5651,7 +5625,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5686,7 +5660,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5721,7 +5695,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5756,7 +5730,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5791,7 +5765,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5826,7 +5800,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5861,7 +5835,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5896,7 +5870,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5931,7 +5905,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5966,7 +5940,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -6001,7 +5975,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6036,7 +6010,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6071,7 +6045,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6106,7 +6080,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6141,7 +6115,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6176,7 +6150,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6211,7 +6185,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6243,7 +6217,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6275,7 +6249,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6307,7 +6281,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6339,7 +6313,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6371,7 +6345,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6403,7 +6377,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6435,7 +6409,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6467,7 +6441,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6499,7 +6473,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6531,7 +6505,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6563,7 +6537,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6595,7 +6569,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6627,7 +6601,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6659,7 +6633,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6691,7 +6665,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6723,7 +6697,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6755,7 +6729,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6787,7 +6761,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6819,7 +6793,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6851,7 +6825,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6883,7 +6857,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6915,7 +6889,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6947,7 +6921,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6979,7 +6953,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -7011,7 +6985,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7043,7 +7017,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7075,7 +7049,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7107,7 +7081,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7139,7 +7113,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7171,7 +7145,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7203,7 +7177,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7235,7 +7209,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7267,7 +7241,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7299,7 +7273,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7331,7 +7305,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7363,7 +7337,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7395,7 +7369,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7427,7 +7401,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7459,7 +7433,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7491,7 +7465,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="2">
+      <c r="J185" s="1">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7523,7 +7497,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="2">
+      <c r="J186" s="1">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7555,7 +7529,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="2">
+      <c r="J187" s="1">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7587,7 +7561,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="2">
+      <c r="J188" s="1">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7619,7 +7593,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="2">
+      <c r="J189" s="1">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7651,7 +7625,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="2">
+      <c r="J190" s="1">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7683,7 +7657,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="2">
+      <c r="J191" s="1">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7715,7 +7689,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="2">
+      <c r="J192" s="1">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7747,7 +7721,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="2">
+      <c r="J193" s="1">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7779,7 +7753,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="2">
+      <c r="J194" s="1">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (17/09/2026 12:58)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1019,8 +1019,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1036,7 +1044,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1044,12 +1052,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1349,37 +1375,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1408,7 +1434,7 @@
       <c r="H2">
         <v>-4300.3</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1440,7 +1466,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1472,7 +1498,7 @@
       <c r="H4">
         <v>-910.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1504,7 +1530,7 @@
       <c r="H5">
         <v>-868</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1536,7 +1562,7 @@
       <c r="H6">
         <v>-483.8</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1568,7 +1594,7 @@
       <c r="H7">
         <v>-417</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46014</v>
       </c>
       <c r="K7" t="b">
@@ -1600,7 +1626,7 @@
       <c r="H8">
         <v>-414.2</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1632,7 +1658,7 @@
       <c r="H9">
         <v>-391.8</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>42769</v>
       </c>
       <c r="K9" t="b">
@@ -1664,7 +1690,7 @@
       <c r="H10">
         <v>-391.6</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>45804</v>
       </c>
       <c r="K10" t="b">
@@ -1696,7 +1722,7 @@
       <c r="H11">
         <v>-391.6</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>45804</v>
       </c>
       <c r="K11" t="b">
@@ -1728,7 +1754,7 @@
       <c r="H12">
         <v>-372.9</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42821</v>
       </c>
       <c r="K12" t="b">
@@ -1760,7 +1786,7 @@
       <c r="H13">
         <v>-372.9</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46014</v>
       </c>
       <c r="K13" t="b">
@@ -1792,7 +1818,7 @@
       <c r="H14">
         <v>-372.9</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46014</v>
       </c>
       <c r="K14" t="b">
@@ -1824,7 +1850,7 @@
       <c r="H15">
         <v>-372.9</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46014</v>
       </c>
       <c r="K15" t="b">
@@ -1856,7 +1882,7 @@
       <c r="H16">
         <v>-367.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46017</v>
       </c>
       <c r="K16" t="b">
@@ -1888,7 +1914,7 @@
       <c r="H17">
         <v>-367.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46017</v>
       </c>
       <c r="K17" t="b">
@@ -1920,7 +1946,7 @@
       <c r="H18">
         <v>-347.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>40979</v>
       </c>
       <c r="K18" t="b">
@@ -1952,7 +1978,7 @@
       <c r="H19">
         <v>-293.8</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>45846</v>
       </c>
       <c r="K19" t="b">
@@ -1984,7 +2010,7 @@
       <c r="H20">
         <v>-206.4</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>36669</v>
       </c>
       <c r="K20" t="b">
@@ -2016,7 +2042,7 @@
       <c r="H21">
         <v>-131.6</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46111</v>
       </c>
       <c r="K21" t="b">
@@ -2048,7 +2074,7 @@
       <c r="H22">
         <v>-131.6</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46111</v>
       </c>
       <c r="K22" t="b">
@@ -2080,7 +2106,7 @@
       <c r="H23">
         <v>-131.6</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46111</v>
       </c>
       <c r="K23" t="b">
@@ -2112,7 +2138,7 @@
       <c r="H24">
         <v>-131.6</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46111</v>
       </c>
       <c r="K24" t="b">
@@ -2144,7 +2170,7 @@
       <c r="H25">
         <v>-131.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46111</v>
       </c>
       <c r="K25" t="b">
@@ -2176,7 +2202,7 @@
       <c r="H26">
         <v>-98.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>41204</v>
       </c>
       <c r="K26" t="b">
@@ -2208,7 +2234,7 @@
       <c r="H27">
         <v>-47.2</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>44011</v>
       </c>
       <c r="K27" t="b">
@@ -2240,7 +2266,7 @@
       <c r="H28">
         <v>-22.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46226</v>
       </c>
       <c r="K28" t="b">
@@ -2272,7 +2298,7 @@
       <c r="H29">
         <v>4.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46265</v>
       </c>
       <c r="K29" t="b">
@@ -2304,7 +2330,7 @@
       <c r="H30">
         <v>7.5</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46265</v>
       </c>
       <c r="K30" t="b">
@@ -2336,7 +2362,7 @@
       <c r="H31">
         <v>10</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46265</v>
       </c>
       <c r="K31" t="b">
@@ -2368,7 +2394,7 @@
       <c r="H32">
         <v>12.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46265</v>
       </c>
       <c r="K32" t="b">
@@ -2400,7 +2426,7 @@
       <c r="H33">
         <v>14</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46265</v>
       </c>
       <c r="K33" t="b">
@@ -2432,7 +2458,7 @@
       <c r="H34">
         <v>17.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46265</v>
       </c>
       <c r="K34" t="b">
@@ -2464,7 +2490,7 @@
       <c r="H35">
         <v>20.4</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46265</v>
       </c>
       <c r="K35" t="b">
@@ -2496,7 +2522,7 @@
       <c r="H36">
         <v>21.2</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46265</v>
       </c>
       <c r="K36" t="b">
@@ -2528,7 +2554,7 @@
       <c r="H37">
         <v>26.2</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46265</v>
       </c>
       <c r="K37" t="b">
@@ -2560,7 +2586,7 @@
       <c r="H38">
         <v>33.6</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46364</v>
       </c>
       <c r="K38" t="b">
@@ -2592,7 +2618,7 @@
       <c r="H39">
         <v>42.2</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46269</v>
       </c>
       <c r="K39" t="b">
@@ -2624,7 +2650,7 @@
       <c r="H40">
         <v>42.8</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46291</v>
       </c>
       <c r="K40" t="b">
@@ -2656,7 +2682,7 @@
       <c r="H41">
         <v>45.7</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46395</v>
       </c>
       <c r="K41" t="b">
@@ -2688,7 +2714,7 @@
       <c r="H42">
         <v>47.2</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46280</v>
       </c>
       <c r="K42" t="b">
@@ -2720,7 +2746,7 @@
       <c r="H43">
         <v>48.7</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46281</v>
       </c>
       <c r="K43" t="b">
@@ -2752,7 +2778,7 @@
       <c r="H44">
         <v>60</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46281</v>
       </c>
       <c r="K44" t="b">
@@ -2784,7 +2810,7 @@
       <c r="H45">
         <v>62.6</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46265</v>
       </c>
       <c r="K45" t="b">
@@ -2816,7 +2842,7 @@
       <c r="H46">
         <v>64.59999999999999</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46265</v>
       </c>
       <c r="K46" t="b">
@@ -2848,7 +2874,7 @@
       <c r="H47">
         <v>67.59999999999999</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46267</v>
       </c>
       <c r="K47" t="b">
@@ -2880,7 +2906,7 @@
       <c r="H48">
         <v>68.3</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46278</v>
       </c>
       <c r="K48" t="b">
@@ -2912,7 +2938,7 @@
       <c r="H49">
         <v>69.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46453</v>
       </c>
       <c r="K49" t="b">
@@ -2944,7 +2970,7 @@
       <c r="H50">
         <v>69.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46265</v>
       </c>
       <c r="K50" t="b">
@@ -2976,7 +3002,7 @@
       <c r="H51">
         <v>69.8</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46265</v>
       </c>
       <c r="K51" t="b">
@@ -3008,7 +3034,7 @@
       <c r="H52">
         <v>72.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46275</v>
       </c>
       <c r="K52" t="b">
@@ -3040,7 +3066,7 @@
       <c r="H53">
         <v>72.2</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46275</v>
       </c>
       <c r="K53" t="b">
@@ -3072,7 +3098,7 @@
       <c r="H54">
         <v>78.09999999999999</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46265</v>
       </c>
       <c r="K54" t="b">
@@ -3104,7 +3130,7 @@
       <c r="H55">
         <v>82.8</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46487</v>
       </c>
       <c r="K55" t="b">
@@ -3136,7 +3162,7 @@
       <c r="H56">
         <v>83.09999999999999</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46285</v>
       </c>
       <c r="K56" t="b">
@@ -3168,7 +3194,7 @@
       <c r="H57">
         <v>84.8</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46492</v>
       </c>
       <c r="K57" t="b">
@@ -3200,7 +3226,7 @@
       <c r="H58">
         <v>104.9</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46297</v>
       </c>
       <c r="K58" t="b">
@@ -3232,7 +3258,7 @@
       <c r="H59">
         <v>107.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46283</v>
       </c>
       <c r="K59" t="b">
@@ -3264,7 +3290,7 @@
       <c r="H60">
         <v>111.9</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46300</v>
       </c>
       <c r="K60" t="b">
@@ -3296,7 +3322,7 @@
       <c r="H61">
         <v>111.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46300</v>
       </c>
       <c r="K61" t="b">
@@ -3328,7 +3354,7 @@
       <c r="H62">
         <v>111.9</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46300</v>
       </c>
       <c r="K62" t="b">
@@ -3360,7 +3386,7 @@
       <c r="H63">
         <v>111.9</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46300</v>
       </c>
       <c r="K63" t="b">
@@ -3392,7 +3418,7 @@
       <c r="H64">
         <v>111.9</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46300</v>
       </c>
       <c r="K64" t="b">
@@ -3424,7 +3450,7 @@
       <c r="H65">
         <v>128.8</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>46308</v>
       </c>
       <c r="K65" t="b">
@@ -3456,7 +3482,7 @@
       <c r="H66">
         <v>131.1</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>46336</v>
       </c>
       <c r="K66" t="b">
@@ -3488,7 +3514,7 @@
       <c r="H67">
         <v>138.4</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>46343</v>
       </c>
       <c r="K67" t="b">
@@ -3520,7 +3546,7 @@
       <c r="H68">
         <v>141</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46350</v>
       </c>
       <c r="K68" t="b">
@@ -3552,7 +3578,7 @@
       <c r="H69">
         <v>162</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46391</v>
       </c>
       <c r="K69" t="b">
@@ -3584,7 +3610,7 @@
       <c r="H70">
         <v>167.2</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46330</v>
       </c>
       <c r="K70" t="b">
@@ -3616,7 +3642,7 @@
       <c r="H71">
         <v>177.4</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46418</v>
       </c>
       <c r="K71" t="b">
@@ -3648,7 +3674,7 @@
       <c r="H72">
         <v>200</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46356</v>
       </c>
       <c r="K72" t="b">
@@ -3680,7 +3706,7 @@
       <c r="H73">
         <v>203.6</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46436</v>
       </c>
       <c r="K73" t="b">
@@ -3712,7 +3738,7 @@
       <c r="H74">
         <v>221.2</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46426</v>
       </c>
       <c r="K74" t="b">
@@ -3744,7 +3770,7 @@
       <c r="H75">
         <v>240.8</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46450</v>
       </c>
       <c r="K75" t="b">
@@ -3776,7 +3802,7 @@
       <c r="H76">
         <v>245.8</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46452</v>
       </c>
       <c r="K76" t="b">
@@ -3808,7 +3834,7 @@
       <c r="H77">
         <v>263.4</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46322</v>
       </c>
       <c r="K77" t="b">
@@ -3840,7 +3866,7 @@
       <c r="H78">
         <v>275.2</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46433</v>
       </c>
       <c r="K78" t="b">
@@ -3875,7 +3901,7 @@
       <c r="I79" t="s">
         <v>311</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>36557</v>
       </c>
       <c r="K79" t="b">
@@ -3910,7 +3936,7 @@
       <c r="I80" t="s">
         <v>312</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>41275</v>
       </c>
       <c r="K80" t="b">
@@ -3945,7 +3971,7 @@
       <c r="I81" t="s">
         <v>313</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>45380</v>
       </c>
       <c r="K81" t="b">
@@ -3980,7 +4006,7 @@
       <c r="I82" t="s">
         <v>314</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>45421</v>
       </c>
       <c r="K82" t="b">
@@ -4015,7 +4041,7 @@
       <c r="I83" t="s">
         <v>314</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>45428</v>
       </c>
       <c r="K83" t="b">
@@ -4050,7 +4076,7 @@
       <c r="I84" t="s">
         <v>315</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>45490</v>
       </c>
       <c r="K84" t="b">
@@ -4085,7 +4111,7 @@
       <c r="I85" t="s">
         <v>316</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>45566</v>
       </c>
       <c r="K85" t="b">
@@ -4120,7 +4146,7 @@
       <c r="I86" t="s">
         <v>317</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>45986</v>
       </c>
       <c r="K86" t="b">
@@ -4155,7 +4181,7 @@
       <c r="I87" t="s">
         <v>318</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46284</v>
       </c>
       <c r="K87" t="b">
@@ -4190,7 +4216,7 @@
       <c r="I88" t="s">
         <v>319</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46305</v>
       </c>
       <c r="K88" t="b">
@@ -4225,7 +4251,7 @@
       <c r="I89" t="s">
         <v>319</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46310</v>
       </c>
       <c r="K89" t="b">
@@ -4260,7 +4286,7 @@
       <c r="I90" t="s">
         <v>319</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46317</v>
       </c>
       <c r="K90" t="b">
@@ -4295,7 +4321,7 @@
       <c r="I91" t="s">
         <v>319</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46319</v>
       </c>
       <c r="K91" t="b">
@@ -4330,7 +4356,7 @@
       <c r="I92" t="s">
         <v>320</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46333</v>
       </c>
       <c r="K92" t="b">
@@ -4365,7 +4391,7 @@
       <c r="I93" t="s">
         <v>320</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46338</v>
       </c>
       <c r="K93" t="b">
@@ -4400,7 +4426,7 @@
       <c r="I94" t="s">
         <v>320</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46338</v>
       </c>
       <c r="K94" t="b">
@@ -4435,7 +4461,7 @@
       <c r="I95" t="s">
         <v>320</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46341</v>
       </c>
       <c r="K95" t="b">
@@ -4470,7 +4496,7 @@
       <c r="I96" t="s">
         <v>320</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46344</v>
       </c>
       <c r="K96" t="b">
@@ -4505,7 +4531,7 @@
       <c r="I97" t="s">
         <v>321</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46360</v>
       </c>
       <c r="K97" t="b">
@@ -4540,7 +4566,7 @@
       <c r="I98" t="s">
         <v>321</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46360</v>
       </c>
       <c r="K98" t="b">
@@ -4575,7 +4601,7 @@
       <c r="I99" t="s">
         <v>321</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46367</v>
       </c>
       <c r="K99" t="b">
@@ -4610,7 +4636,7 @@
       <c r="I100" t="s">
         <v>321</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46375</v>
       </c>
       <c r="K100" t="b">
@@ -4645,7 +4671,7 @@
       <c r="I101" t="s">
         <v>321</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46387</v>
       </c>
       <c r="K101" t="b">
@@ -4680,7 +4706,7 @@
       <c r="I102" t="s">
         <v>321</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46387</v>
       </c>
       <c r="K102" t="b">
@@ -4715,7 +4741,7 @@
       <c r="I103" t="s">
         <v>321</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46387</v>
       </c>
       <c r="K103" t="b">
@@ -4750,7 +4776,7 @@
       <c r="I104" t="s">
         <v>321</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46388</v>
       </c>
       <c r="K104" t="b">
@@ -4785,7 +4811,7 @@
       <c r="I105" t="s">
         <v>322</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46401</v>
       </c>
       <c r="K105" t="b">
@@ -4820,7 +4846,7 @@
       <c r="I106" t="s">
         <v>322</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46401</v>
       </c>
       <c r="K106" t="b">
@@ -4855,7 +4881,7 @@
       <c r="I107" t="s">
         <v>322</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46401</v>
       </c>
       <c r="K107" t="b">
@@ -4890,7 +4916,7 @@
       <c r="I108" t="s">
         <v>322</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46412</v>
       </c>
       <c r="K108" t="b">
@@ -4925,7 +4951,7 @@
       <c r="I109" t="s">
         <v>322</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46412</v>
       </c>
       <c r="K109" t="b">
@@ -4960,7 +4986,7 @@
       <c r="I110" t="s">
         <v>322</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46412</v>
       </c>
       <c r="K110" t="b">
@@ -4995,7 +5021,7 @@
       <c r="I111" t="s">
         <v>323</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46424</v>
       </c>
       <c r="K111" t="b">
@@ -5030,7 +5056,7 @@
       <c r="I112" t="s">
         <v>323</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46437</v>
       </c>
       <c r="K112" t="b">
@@ -5065,7 +5091,7 @@
       <c r="I113" t="s">
         <v>323</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46451</v>
       </c>
       <c r="K113" t="b">
@@ -5100,7 +5126,7 @@
       <c r="I114" t="s">
         <v>323</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46451</v>
       </c>
       <c r="K114" t="b">
@@ -5135,7 +5161,7 @@
       <c r="I115" t="s">
         <v>324</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46455</v>
       </c>
       <c r="K115" t="b">
@@ -5170,7 +5196,7 @@
       <c r="I116" t="s">
         <v>324</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46456</v>
       </c>
       <c r="K116" t="b">
@@ -5205,7 +5231,7 @@
       <c r="I117" t="s">
         <v>324</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46457</v>
       </c>
       <c r="K117" t="b">
@@ -5240,7 +5266,7 @@
       <c r="I118" t="s">
         <v>324</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46464</v>
       </c>
       <c r="K118" t="b">
@@ -5275,7 +5301,7 @@
       <c r="I119" t="s">
         <v>324</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46470</v>
       </c>
       <c r="K119" t="b">
@@ -5310,7 +5336,7 @@
       <c r="I120" t="s">
         <v>325</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46485</v>
       </c>
       <c r="K120" t="b">
@@ -5345,7 +5371,7 @@
       <c r="I121" t="s">
         <v>325</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46499</v>
       </c>
       <c r="K121" t="b">
@@ -5380,7 +5406,7 @@
       <c r="I122" t="s">
         <v>325</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46504</v>
       </c>
       <c r="K122" t="b">
@@ -5415,7 +5441,7 @@
       <c r="I123" t="s">
         <v>325</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46504</v>
       </c>
       <c r="K123" t="b">
@@ -5450,7 +5476,7 @@
       <c r="I124" t="s">
         <v>325</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46507</v>
       </c>
       <c r="K124" t="b">
@@ -5485,7 +5511,7 @@
       <c r="I125" t="s">
         <v>325</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46508</v>
       </c>
       <c r="K125" t="b">
@@ -5520,7 +5546,7 @@
       <c r="I126" t="s">
         <v>325</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46512</v>
       </c>
       <c r="K126" t="b">
@@ -5555,7 +5581,7 @@
       <c r="I127" t="s">
         <v>326</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46512</v>
       </c>
       <c r="K127" t="b">
@@ -5590,7 +5616,7 @@
       <c r="I128" t="s">
         <v>326</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46528</v>
       </c>
       <c r="K128" t="b">
@@ -5625,7 +5651,7 @@
       <c r="I129" t="s">
         <v>326</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46529</v>
       </c>
       <c r="K129" t="b">
@@ -5660,7 +5686,7 @@
       <c r="I130" t="s">
         <v>326</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46537</v>
       </c>
       <c r="K130" t="b">
@@ -5695,7 +5721,7 @@
       <c r="I131" t="s">
         <v>327</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46546</v>
       </c>
       <c r="K131" t="b">
@@ -5730,7 +5756,7 @@
       <c r="I132" t="s">
         <v>327</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46547</v>
       </c>
       <c r="K132" t="b">
@@ -5765,7 +5791,7 @@
       <c r="I133" t="s">
         <v>327</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46547</v>
       </c>
       <c r="K133" t="b">
@@ -5800,7 +5826,7 @@
       <c r="I134" t="s">
         <v>327</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46547</v>
       </c>
       <c r="K134" t="b">
@@ -5835,7 +5861,7 @@
       <c r="I135" t="s">
         <v>327</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46551</v>
       </c>
       <c r="K135" t="b">
@@ -5870,7 +5896,7 @@
       <c r="I136" t="s">
         <v>327</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46560</v>
       </c>
       <c r="K136" t="b">
@@ -5905,7 +5931,7 @@
       <c r="I137" t="s">
         <v>327</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46564</v>
       </c>
       <c r="K137" t="b">
@@ -5940,7 +5966,7 @@
       <c r="I138" t="s">
         <v>327</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46567</v>
       </c>
       <c r="K138" t="b">
@@ -5975,7 +6001,7 @@
       <c r="I139" t="s">
         <v>327</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46568</v>
       </c>
       <c r="K139" t="b">
@@ -6010,7 +6036,7 @@
       <c r="I140" t="s">
         <v>328</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46578</v>
       </c>
       <c r="K140" t="b">
@@ -6045,7 +6071,7 @@
       <c r="I141" t="s">
         <v>328</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46592</v>
       </c>
       <c r="K141" t="b">
@@ -6080,7 +6106,7 @@
       <c r="I142" t="s">
         <v>328</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46592</v>
       </c>
       <c r="K142" t="b">
@@ -6115,7 +6141,7 @@
       <c r="I143" t="s">
         <v>329</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46212</v>
       </c>
       <c r="K143" t="b">
@@ -6150,7 +6176,7 @@
       <c r="I144" t="s">
         <v>330</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46225</v>
       </c>
       <c r="K144" t="b">
@@ -6185,7 +6211,7 @@
       <c r="I145" t="s">
         <v>331</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46263</v>
       </c>
       <c r="K145" t="b">
@@ -6217,7 +6243,7 @@
       <c r="H146">
         <v>-1476</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>43773</v>
       </c>
       <c r="K146" t="b">
@@ -6249,7 +6275,7 @@
       <c r="H147">
         <v>-1469</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>43773</v>
       </c>
       <c r="K147" t="b">
@@ -6281,7 +6307,7 @@
       <c r="H148">
         <v>-1186</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>45295</v>
       </c>
       <c r="K148" t="b">
@@ -6313,7 +6339,7 @@
       <c r="H149">
         <v>-1048</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>45617</v>
       </c>
       <c r="K149" t="b">
@@ -6345,7 +6371,7 @@
       <c r="H150">
         <v>-980</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>45677</v>
       </c>
       <c r="K150" t="b">
@@ -6377,7 +6403,7 @@
       <c r="H151">
         <v>-961</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>44944</v>
       </c>
       <c r="K151" t="b">
@@ -6409,7 +6435,7 @@
       <c r="H152">
         <v>-252</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46092</v>
       </c>
       <c r="K152" t="b">
@@ -6441,7 +6467,7 @@
       <c r="H153">
         <v>3</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46265</v>
       </c>
       <c r="K153" t="b">
@@ -6473,7 +6499,7 @@
       <c r="H154">
         <v>3</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46265</v>
       </c>
       <c r="K154" t="b">
@@ -6505,7 +6531,7 @@
       <c r="H155">
         <v>43</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46440</v>
       </c>
       <c r="K155" t="b">
@@ -6537,7 +6563,7 @@
       <c r="H156">
         <v>43</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46440</v>
       </c>
       <c r="K156" t="b">
@@ -6569,7 +6595,7 @@
       <c r="H157">
         <v>72</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46289</v>
       </c>
       <c r="K157" t="b">
@@ -6601,7 +6627,7 @@
       <c r="H158">
         <v>72</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46289</v>
       </c>
       <c r="K158" t="b">
@@ -6633,7 +6659,7 @@
       <c r="H159">
         <v>81</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46405</v>
       </c>
       <c r="K159" t="b">
@@ -6665,7 +6691,7 @@
       <c r="H160">
         <v>102</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46463</v>
       </c>
       <c r="K160" t="b">
@@ -6697,7 +6723,7 @@
       <c r="H161">
         <v>109</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46353</v>
       </c>
       <c r="K161" t="b">
@@ -6729,7 +6755,7 @@
       <c r="H162">
         <v>127</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46417</v>
       </c>
       <c r="K162" t="b">
@@ -6761,7 +6787,7 @@
       <c r="H163">
         <v>152</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46271</v>
       </c>
       <c r="K163" t="b">
@@ -6793,7 +6819,7 @@
       <c r="H164">
         <v>152</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46271</v>
       </c>
       <c r="K164" t="b">
@@ -6825,7 +6851,7 @@
       <c r="H165">
         <v>153</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46458</v>
       </c>
       <c r="K165" t="b">
@@ -6857,7 +6883,7 @@
       <c r="H166">
         <v>158</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46381</v>
       </c>
       <c r="K166" t="b">
@@ -6889,7 +6915,7 @@
       <c r="H167">
         <v>163</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46592</v>
       </c>
       <c r="K167" t="b">
@@ -6921,7 +6947,7 @@
       <c r="H168">
         <v>167</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46441</v>
       </c>
       <c r="K168" t="b">
@@ -6953,7 +6979,7 @@
       <c r="H169">
         <v>169</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46391</v>
       </c>
       <c r="K169" t="b">
@@ -6985,7 +7011,7 @@
       <c r="H170">
         <v>184</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46385</v>
       </c>
       <c r="K170" t="b">
@@ -7017,7 +7043,7 @@
       <c r="H171">
         <v>186</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46387</v>
       </c>
       <c r="K171" t="b">
@@ -7049,7 +7075,7 @@
       <c r="H172">
         <v>206</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46399</v>
       </c>
       <c r="K172" t="b">
@@ -7081,7 +7107,7 @@
       <c r="H173">
         <v>206</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46399</v>
       </c>
       <c r="K173" t="b">
@@ -7113,7 +7139,7 @@
       <c r="H174">
         <v>234</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46458</v>
       </c>
       <c r="K174" t="b">
@@ -7145,7 +7171,7 @@
       <c r="H175">
         <v>248</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46528</v>
       </c>
       <c r="K175" t="b">
@@ -7177,7 +7203,7 @@
       <c r="H176">
         <v>317</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46540</v>
       </c>
       <c r="K176" t="b">
@@ -7209,7 +7235,7 @@
       <c r="H177">
         <v>340</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46547</v>
       </c>
       <c r="K177" t="b">
@@ -7241,7 +7267,7 @@
       <c r="H178">
         <v>364</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46557</v>
       </c>
       <c r="K178" t="b">
@@ -7273,7 +7299,7 @@
       <c r="H179">
         <v>368</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46571</v>
       </c>
       <c r="K179" t="b">
@@ -7305,7 +7331,7 @@
       <c r="H180">
         <v>368</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46571</v>
       </c>
       <c r="K180" t="b">
@@ -7337,7 +7363,7 @@
       <c r="H181">
         <v>370</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46562</v>
       </c>
       <c r="K181" t="b">
@@ -7369,7 +7395,7 @@
       <c r="H182">
         <v>385</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46574</v>
       </c>
       <c r="K182" t="b">
@@ -7401,7 +7427,7 @@
       <c r="H183">
         <v>385</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46574</v>
       </c>
       <c r="K183" t="b">
@@ -7433,7 +7459,7 @@
       <c r="H184">
         <v>417</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46578</v>
       </c>
       <c r="K184" t="b">
@@ -7465,7 +7491,7 @@
       <c r="H185">
         <v>721</v>
       </c>
-      <c r="J185" s="1">
+      <c r="J185" s="2">
         <v>46345</v>
       </c>
       <c r="K185" t="b">
@@ -7497,7 +7523,7 @@
       <c r="H186">
         <v>721</v>
       </c>
-      <c r="J186" s="1">
+      <c r="J186" s="2">
         <v>46345</v>
       </c>
       <c r="K186" t="b">
@@ -7529,7 +7555,7 @@
       <c r="H187">
         <v>850</v>
       </c>
-      <c r="J187" s="1">
+      <c r="J187" s="2">
         <v>46366</v>
       </c>
       <c r="K187" t="b">
@@ -7561,7 +7587,7 @@
       <c r="H188">
         <v>850</v>
       </c>
-      <c r="J188" s="1">
+      <c r="J188" s="2">
         <v>46366</v>
       </c>
       <c r="K188" t="b">
@@ -7593,7 +7619,7 @@
       <c r="H189">
         <v>1661</v>
       </c>
-      <c r="J189" s="1">
+      <c r="J189" s="2">
         <v>46524</v>
       </c>
       <c r="K189" t="b">
@@ -7625,7 +7651,7 @@
       <c r="H190">
         <v>1661</v>
       </c>
-      <c r="J190" s="1">
+      <c r="J190" s="2">
         <v>46524</v>
       </c>
       <c r="K190" t="b">
@@ -7657,7 +7683,7 @@
       <c r="H191">
         <v>488</v>
       </c>
-      <c r="J191" s="1">
+      <c r="J191" s="2">
         <v>46190</v>
       </c>
       <c r="K191" t="b">
@@ -7689,7 +7715,7 @@
       <c r="H192">
         <v>25565</v>
       </c>
-      <c r="J192" s="1">
+      <c r="J192" s="2">
         <v>46190</v>
       </c>
       <c r="K192" t="b">
@@ -7721,7 +7747,7 @@
       <c r="H193">
         <v>25567</v>
       </c>
-      <c r="J193" s="1">
+      <c r="J193" s="2">
         <v>46190</v>
       </c>
       <c r="K193" t="b">
@@ -7753,7 +7779,7 @@
       <c r="H194">
         <v>31293</v>
       </c>
-      <c r="J194" s="1">
+      <c r="J194" s="2">
         <v>46190</v>
       </c>
       <c r="K194" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (18/09/2026 16:37)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (21/09/2026 13:59)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (21/09/2026 14:30)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (22/09/2026 12:30)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (23/09/2026 10:03)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (23/09/2026 12:26)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (28/09/2026 13:06)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (28/09/2026 15:35)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (29/09/2026 19:54)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (30/09/2026 13:48)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (30/09/2026 15:55)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (01/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (02/10/2026 09:56)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (02/10/2026 13:37)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (05/10/2026 08:40)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (06/10/2026 14:09)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (07/10/2026 11:10)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,8 +953,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -970,7 +978,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -978,12 +986,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1283,37 +1309,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1342,7 +1368,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1374,7 +1400,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1406,7 +1432,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1438,7 +1464,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1470,7 +1496,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1502,7 +1528,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1534,7 +1560,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1566,7 +1592,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1598,7 +1624,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1630,7 +1656,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1662,7 +1688,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1694,7 +1720,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1726,7 +1752,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1758,7 +1784,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1790,7 +1816,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1822,7 +1848,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1854,7 +1880,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1886,7 +1912,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1918,7 +1944,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1950,7 +1976,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -1982,7 +2008,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2014,7 +2040,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2046,7 +2072,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2078,7 +2104,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2110,7 +2136,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2142,7 +2168,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2174,7 +2200,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2206,7 +2232,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2238,7 +2264,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2270,7 +2296,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2302,7 +2328,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2334,7 +2360,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2366,7 +2392,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2398,7 +2424,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2430,7 +2456,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2462,7 +2488,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2494,7 +2520,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2526,7 +2552,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2558,7 +2584,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2590,7 +2616,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2622,7 +2648,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2654,7 +2680,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2686,7 +2712,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2718,7 +2744,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2750,7 +2776,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2782,7 +2808,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2814,7 +2840,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2846,7 +2872,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2878,7 +2904,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2910,7 +2936,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2942,7 +2968,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -2974,7 +3000,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3006,7 +3032,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3038,7 +3064,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3070,7 +3096,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3102,7 +3128,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3134,7 +3160,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3166,7 +3192,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3201,7 +3227,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3236,7 +3262,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3271,7 +3297,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3306,7 +3332,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3341,7 +3367,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3376,7 +3402,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3411,7 +3437,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3446,7 +3472,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3481,7 +3507,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3516,7 +3542,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3551,7 +3577,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3586,7 +3612,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3621,7 +3647,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3656,7 +3682,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3691,7 +3717,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3726,7 +3752,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3761,7 +3787,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3796,7 +3822,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3831,7 +3857,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3866,7 +3892,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3901,7 +3927,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3936,7 +3962,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3971,7 +3997,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4006,7 +4032,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4041,7 +4067,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4076,7 +4102,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4111,7 +4137,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4146,7 +4172,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4181,7 +4207,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4216,7 +4242,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4251,7 +4277,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4286,7 +4312,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4321,7 +4347,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4356,7 +4382,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4391,7 +4417,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4426,7 +4452,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4461,7 +4487,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4496,7 +4522,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4531,7 +4557,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4566,7 +4592,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4601,7 +4627,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4636,7 +4662,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4671,7 +4697,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4706,7 +4732,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4741,7 +4767,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4776,7 +4802,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4811,7 +4837,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4846,7 +4872,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4881,7 +4907,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4916,7 +4942,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4951,7 +4977,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -4986,7 +5012,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5021,7 +5047,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5056,7 +5082,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5091,7 +5117,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5126,7 +5152,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5161,7 +5187,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5196,7 +5222,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5231,7 +5257,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5266,7 +5292,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5301,7 +5327,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5336,7 +5362,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5371,7 +5397,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5406,7 +5432,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5441,7 +5467,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5476,7 +5502,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5508,7 +5534,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5540,7 +5566,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5572,7 +5598,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5604,7 +5630,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5636,7 +5662,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5668,7 +5694,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5700,7 +5726,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5732,7 +5758,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5764,7 +5790,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5796,7 +5822,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5828,7 +5854,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5860,7 +5886,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5892,7 +5918,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5924,7 +5950,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5956,7 +5982,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -5988,7 +6014,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6020,7 +6046,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6052,7 +6078,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6084,7 +6110,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6116,7 +6142,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6148,7 +6174,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6180,7 +6206,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6212,7 +6238,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6244,7 +6270,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6276,7 +6302,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6308,7 +6334,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6340,7 +6366,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6372,7 +6398,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6404,7 +6430,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6436,7 +6462,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6468,7 +6494,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6500,7 +6526,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6532,7 +6558,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6564,7 +6590,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6596,7 +6622,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6628,7 +6654,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6660,7 +6686,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6692,7 +6718,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6724,7 +6750,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6756,7 +6782,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6788,7 +6814,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6820,7 +6846,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6852,7 +6878,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6884,7 +6910,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (07/10/2026 14:47)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -953,16 +953,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -978,7 +970,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -986,30 +978,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1309,37 +1283,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1368,7 +1342,7 @@
       <c r="H2">
         <v>-4349.4</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>39285</v>
       </c>
       <c r="K2" t="b">
@@ -1400,7 +1374,7 @@
       <c r="H3">
         <v>-2354.2</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1432,7 +1406,7 @@
       <c r="H4">
         <v>-922.4</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>40669</v>
       </c>
       <c r="K4" t="b">
@@ -1464,7 +1438,7 @@
       <c r="H5">
         <v>-879.8</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>44884</v>
       </c>
       <c r="K5" t="b">
@@ -1496,7 +1470,7 @@
       <c r="H6">
         <v>-536.4</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>43855</v>
       </c>
       <c r="K6" t="b">
@@ -1528,7 +1502,7 @@
       <c r="H7">
         <v>-484.3</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1560,7 +1534,7 @@
       <c r="H8">
         <v>-482.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>45804</v>
       </c>
       <c r="K8" t="b">
@@ -1592,7 +1566,7 @@
       <c r="H9">
         <v>-466.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1624,7 +1598,7 @@
       <c r="H10">
         <v>-463.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>40979</v>
       </c>
       <c r="K10" t="b">
@@ -1656,7 +1630,7 @@
       <c r="H11">
         <v>-463.3</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46014</v>
       </c>
       <c r="K11" t="b">
@@ -1688,7 +1662,7 @@
       <c r="H12">
         <v>-391.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>42769</v>
       </c>
       <c r="K12" t="b">
@@ -1720,7 +1694,7 @@
       <c r="H13">
         <v>-390</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>32786</v>
       </c>
       <c r="K13" t="b">
@@ -1752,7 +1726,7 @@
       <c r="H14">
         <v>-211.2</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>34700</v>
       </c>
       <c r="K14" t="b">
@@ -1784,7 +1758,7 @@
       <c r="H15">
         <v>-176</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>41204</v>
       </c>
       <c r="K15" t="b">
@@ -1816,7 +1790,7 @@
       <c r="H16">
         <v>-159.2</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1848,7 +1822,7 @@
       <c r="H17">
         <v>-159.2</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1880,7 +1854,7 @@
       <c r="H18">
         <v>-159.2</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1912,7 +1886,7 @@
       <c r="H19">
         <v>-159.2</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46111</v>
       </c>
       <c r="K19" t="b">
@@ -1944,7 +1918,7 @@
       <c r="H20">
         <v>-101.6</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46161</v>
       </c>
       <c r="K20" t="b">
@@ -1976,7 +1950,7 @@
       <c r="H21">
         <v>-69.7</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46241</v>
       </c>
       <c r="K21" t="b">
@@ -2008,7 +1982,7 @@
       <c r="H22">
         <v>-61.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46242</v>
       </c>
       <c r="K22" t="b">
@@ -2040,7 +2014,7 @@
       <c r="H23">
         <v>-53.5</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46255</v>
       </c>
       <c r="K23" t="b">
@@ -2072,7 +2046,7 @@
       <c r="H24">
         <v>-10</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46276</v>
       </c>
       <c r="K24" t="b">
@@ -2104,7 +2078,7 @@
       <c r="H25">
         <v>-10</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46276</v>
       </c>
       <c r="K25" t="b">
@@ -2136,7 +2110,7 @@
       <c r="H26">
         <v>-7.4</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46269</v>
       </c>
       <c r="K26" t="b">
@@ -2168,7 +2142,7 @@
       <c r="H27">
         <v>-6.3</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46236</v>
       </c>
       <c r="K27" t="b">
@@ -2200,7 +2174,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46282</v>
       </c>
       <c r="K28" t="b">
@@ -2232,7 +2206,7 @@
       <c r="H29">
         <v>7.7</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46295</v>
       </c>
       <c r="K29" t="b">
@@ -2264,7 +2238,7 @@
       <c r="H30">
         <v>9.800000000000001</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46295</v>
       </c>
       <c r="K30" t="b">
@@ -2296,7 +2270,7 @@
       <c r="H31">
         <v>10.9</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46295</v>
       </c>
       <c r="K31" t="b">
@@ -2328,7 +2302,7 @@
       <c r="H32">
         <v>21.8</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46404</v>
       </c>
       <c r="K32" t="b">
@@ -2360,7 +2334,7 @@
       <c r="H33">
         <v>33.9</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46434</v>
       </c>
       <c r="K33" t="b">
@@ -2392,7 +2366,7 @@
       <c r="H34">
         <v>42.8</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46385</v>
       </c>
       <c r="K34" t="b">
@@ -2424,7 +2398,7 @@
       <c r="H35">
         <v>52.7</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46337</v>
       </c>
       <c r="K35" t="b">
@@ -2456,7 +2430,7 @@
       <c r="H36">
         <v>57.5</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46493</v>
       </c>
       <c r="K36" t="b">
@@ -2488,7 +2462,7 @@
       <c r="H37">
         <v>71</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46527</v>
       </c>
       <c r="K37" t="b">
@@ -2520,7 +2494,7 @@
       <c r="H38">
         <v>73</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46532</v>
       </c>
       <c r="K38" t="b">
@@ -2552,7 +2526,7 @@
       <c r="H39">
         <v>82</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46389</v>
       </c>
       <c r="K39" t="b">
@@ -2584,7 +2558,7 @@
       <c r="H40">
         <v>107.1</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46338</v>
       </c>
       <c r="K40" t="b">
@@ -2616,7 +2590,7 @@
       <c r="H41">
         <v>109.8</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46337</v>
       </c>
       <c r="K41" t="b">
@@ -2648,7 +2622,7 @@
       <c r="H42">
         <v>112.9</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46401</v>
       </c>
       <c r="K42" t="b">
@@ -2680,7 +2654,7 @@
       <c r="H43">
         <v>121.9</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46412</v>
       </c>
       <c r="K43" t="b">
@@ -2712,7 +2686,7 @@
       <c r="H44">
         <v>135.1</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46353</v>
       </c>
       <c r="K44" t="b">
@@ -2744,7 +2718,7 @@
       <c r="H45">
         <v>136.2</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46419</v>
       </c>
       <c r="K45" t="b">
@@ -2776,7 +2750,7 @@
       <c r="H46">
         <v>138.8</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46353</v>
       </c>
       <c r="K46" t="b">
@@ -2808,7 +2782,7 @@
       <c r="H47">
         <v>140.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46355</v>
       </c>
       <c r="K47" t="b">
@@ -2840,7 +2814,7 @@
       <c r="H48">
         <v>141.6</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46355</v>
       </c>
       <c r="K48" t="b">
@@ -2872,7 +2846,7 @@
       <c r="H49">
         <v>161.2</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46394</v>
       </c>
       <c r="K49" t="b">
@@ -2904,7 +2878,7 @@
       <c r="H50">
         <v>170.3</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46370</v>
       </c>
       <c r="K50" t="b">
@@ -2936,7 +2910,7 @@
       <c r="H51">
         <v>177.4</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46487</v>
       </c>
       <c r="K51" t="b">
@@ -2968,7 +2942,7 @@
       <c r="H52">
         <v>184.1</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46358</v>
       </c>
       <c r="K52" t="b">
@@ -3000,7 +2974,7 @@
       <c r="H53">
         <v>199.3</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46433</v>
       </c>
       <c r="K53" t="b">
@@ -3032,7 +3006,7 @@
       <c r="H54">
         <v>200</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46367</v>
       </c>
       <c r="K54" t="b">
@@ -3064,7 +3038,7 @@
       <c r="H55">
         <v>203.6</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46388</v>
       </c>
       <c r="K55" t="b">
@@ -3096,7 +3070,7 @@
       <c r="H56">
         <v>207.6</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46391</v>
       </c>
       <c r="K56" t="b">
@@ -3128,7 +3102,7 @@
       <c r="H57">
         <v>226.1</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46442</v>
       </c>
       <c r="K57" t="b">
@@ -3160,7 +3134,7 @@
       <c r="H58">
         <v>277</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46461</v>
       </c>
       <c r="K58" t="b">
@@ -3192,7 +3166,7 @@
       <c r="H59">
         <v>280.6</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46409</v>
       </c>
       <c r="K59" t="b">
@@ -3227,7 +3201,7 @@
       <c r="I60" t="s">
         <v>287</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>36557</v>
       </c>
       <c r="K60" t="b">
@@ -3262,7 +3236,7 @@
       <c r="I61" t="s">
         <v>288</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>41275</v>
       </c>
       <c r="K61" t="b">
@@ -3297,7 +3271,7 @@
       <c r="I62" t="s">
         <v>289</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>45380</v>
       </c>
       <c r="K62" t="b">
@@ -3332,7 +3306,7 @@
       <c r="I63" t="s">
         <v>290</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>45421</v>
       </c>
       <c r="K63" t="b">
@@ -3367,7 +3341,7 @@
       <c r="I64" t="s">
         <v>290</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>45428</v>
       </c>
       <c r="K64" t="b">
@@ -3402,7 +3376,7 @@
       <c r="I65" t="s">
         <v>291</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>45490</v>
       </c>
       <c r="K65" t="b">
@@ -3437,7 +3411,7 @@
       <c r="I66" t="s">
         <v>292</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>45566</v>
       </c>
       <c r="K66" t="b">
@@ -3472,7 +3446,7 @@
       <c r="I67" t="s">
         <v>293</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45986</v>
       </c>
       <c r="K67" t="b">
@@ -3507,7 +3481,7 @@
       <c r="I68" t="s">
         <v>294</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>46197</v>
       </c>
       <c r="K68" t="b">
@@ -3542,7 +3516,7 @@
       <c r="I69" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>46212</v>
       </c>
       <c r="K69" t="b">
@@ -3577,7 +3551,7 @@
       <c r="I70" t="s">
         <v>295</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>46341</v>
       </c>
       <c r="K70" t="b">
@@ -3612,7 +3586,7 @@
       <c r="I71" t="s">
         <v>295</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>46344</v>
       </c>
       <c r="K71" t="b">
@@ -3647,7 +3621,7 @@
       <c r="I72" t="s">
         <v>295</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>46360</v>
       </c>
       <c r="K72" t="b">
@@ -3682,7 +3656,7 @@
       <c r="I73" t="s">
         <v>295</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46367</v>
       </c>
       <c r="K73" t="b">
@@ -3717,7 +3691,7 @@
       <c r="I74" t="s">
         <v>295</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46368</v>
       </c>
       <c r="K74" t="b">
@@ -3752,7 +3726,7 @@
       <c r="I75" t="s">
         <v>295</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46374</v>
       </c>
       <c r="K75" t="b">
@@ -3787,7 +3761,7 @@
       <c r="I76" t="s">
         <v>296</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46375</v>
       </c>
       <c r="K76" t="b">
@@ -3822,7 +3796,7 @@
       <c r="I77" t="s">
         <v>296</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46387</v>
       </c>
       <c r="K77" t="b">
@@ -3857,7 +3831,7 @@
       <c r="I78" t="s">
         <v>296</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46387</v>
       </c>
       <c r="K78" t="b">
@@ -3892,7 +3866,7 @@
       <c r="I79" t="s">
         <v>296</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46387</v>
       </c>
       <c r="K79" t="b">
@@ -3927,7 +3901,7 @@
       <c r="I80" t="s">
         <v>296</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46388</v>
       </c>
       <c r="K80" t="b">
@@ -3962,7 +3936,7 @@
       <c r="I81" t="s">
         <v>296</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46401</v>
       </c>
       <c r="K81" t="b">
@@ -3997,7 +3971,7 @@
       <c r="I82" t="s">
         <v>296</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46401</v>
       </c>
       <c r="K82" t="b">
@@ -4032,7 +4006,7 @@
       <c r="I83" t="s">
         <v>296</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46401</v>
       </c>
       <c r="K83" t="b">
@@ -4067,7 +4041,7 @@
       <c r="I84" t="s">
         <v>297</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46412</v>
       </c>
       <c r="K84" t="b">
@@ -4102,7 +4076,7 @@
       <c r="I85" t="s">
         <v>297</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46412</v>
       </c>
       <c r="K85" t="b">
@@ -4137,7 +4111,7 @@
       <c r="I86" t="s">
         <v>297</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46424</v>
       </c>
       <c r="K86" t="b">
@@ -4172,7 +4146,7 @@
       <c r="I87" t="s">
         <v>297</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46427</v>
       </c>
       <c r="K87" t="b">
@@ -4207,7 +4181,7 @@
       <c r="I88" t="s">
         <v>297</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46427</v>
       </c>
       <c r="K88" t="b">
@@ -4242,7 +4216,7 @@
       <c r="I89" t="s">
         <v>298</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46437</v>
       </c>
       <c r="K89" t="b">
@@ -4277,7 +4251,7 @@
       <c r="I90" t="s">
         <v>298</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46451</v>
       </c>
       <c r="K90" t="b">
@@ -4312,7 +4286,7 @@
       <c r="I91" t="s">
         <v>298</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46451</v>
       </c>
       <c r="K91" t="b">
@@ -4347,7 +4321,7 @@
       <c r="I92" t="s">
         <v>298</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46455</v>
       </c>
       <c r="K92" t="b">
@@ -4382,7 +4356,7 @@
       <c r="I93" t="s">
         <v>298</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46456</v>
       </c>
       <c r="K93" t="b">
@@ -4417,7 +4391,7 @@
       <c r="I94" t="s">
         <v>298</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46457</v>
       </c>
       <c r="K94" t="b">
@@ -4452,7 +4426,7 @@
       <c r="I95" t="s">
         <v>298</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46464</v>
       </c>
       <c r="K95" t="b">
@@ -4487,7 +4461,7 @@
       <c r="I96" t="s">
         <v>299</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46470</v>
       </c>
       <c r="K96" t="b">
@@ -4522,7 +4496,7 @@
       <c r="I97" t="s">
         <v>299</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46485</v>
       </c>
       <c r="K97" t="b">
@@ -4557,7 +4531,7 @@
       <c r="I98" t="s">
         <v>300</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46499</v>
       </c>
       <c r="K98" t="b">
@@ -4592,7 +4566,7 @@
       <c r="I99" t="s">
         <v>300</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46504</v>
       </c>
       <c r="K99" t="b">
@@ -4627,7 +4601,7 @@
       <c r="I100" t="s">
         <v>300</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46507</v>
       </c>
       <c r="K100" t="b">
@@ -4662,7 +4636,7 @@
       <c r="I101" t="s">
         <v>300</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46508</v>
       </c>
       <c r="K101" t="b">
@@ -4697,7 +4671,7 @@
       <c r="I102" t="s">
         <v>300</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46512</v>
       </c>
       <c r="K102" t="b">
@@ -4732,7 +4706,7 @@
       <c r="I103" t="s">
         <v>300</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46512</v>
       </c>
       <c r="K103" t="b">
@@ -4767,7 +4741,7 @@
       <c r="I104" t="s">
         <v>301</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46528</v>
       </c>
       <c r="K104" t="b">
@@ -4802,7 +4776,7 @@
       <c r="I105" t="s">
         <v>301</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46529</v>
       </c>
       <c r="K105" t="b">
@@ -4837,7 +4811,7 @@
       <c r="I106" t="s">
         <v>301</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46537</v>
       </c>
       <c r="K106" t="b">
@@ -4872,7 +4846,7 @@
       <c r="I107" t="s">
         <v>301</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46546</v>
       </c>
       <c r="K107" t="b">
@@ -4907,7 +4881,7 @@
       <c r="I108" t="s">
         <v>301</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46547</v>
       </c>
       <c r="K108" t="b">
@@ -4942,7 +4916,7 @@
       <c r="I109" t="s">
         <v>301</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46547</v>
       </c>
       <c r="K109" t="b">
@@ -4977,7 +4951,7 @@
       <c r="I110" t="s">
         <v>301</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46551</v>
       </c>
       <c r="K110" t="b">
@@ -5012,7 +4986,7 @@
       <c r="I111" t="s">
         <v>302</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46560</v>
       </c>
       <c r="K111" t="b">
@@ -5047,7 +5021,7 @@
       <c r="I112" t="s">
         <v>302</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46567</v>
       </c>
       <c r="K112" t="b">
@@ -5082,7 +5056,7 @@
       <c r="I113" t="s">
         <v>302</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46568</v>
       </c>
       <c r="K113" t="b">
@@ -5117,7 +5091,7 @@
       <c r="I114" t="s">
         <v>302</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46578</v>
       </c>
       <c r="K114" t="b">
@@ -5152,7 +5126,7 @@
       <c r="I115" t="s">
         <v>303</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46592</v>
       </c>
       <c r="K115" t="b">
@@ -5187,7 +5161,7 @@
       <c r="I116" t="s">
         <v>303</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46592</v>
       </c>
       <c r="K116" t="b">
@@ -5222,7 +5196,7 @@
       <c r="I117" t="s">
         <v>303</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46603</v>
       </c>
       <c r="K117" t="b">
@@ -5257,7 +5231,7 @@
       <c r="I118" t="s">
         <v>303</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46611</v>
       </c>
       <c r="K118" t="b">
@@ -5292,7 +5266,7 @@
       <c r="I119" t="s">
         <v>304</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46631</v>
       </c>
       <c r="K119" t="b">
@@ -5327,7 +5301,7 @@
       <c r="I120" t="s">
         <v>304</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46645</v>
       </c>
       <c r="K120" t="b">
@@ -5362,7 +5336,7 @@
       <c r="I121" t="s">
         <v>305</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46254</v>
       </c>
       <c r="K121" t="b">
@@ -5397,7 +5371,7 @@
       <c r="I122" t="s">
         <v>306</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46284</v>
       </c>
       <c r="K122" t="b">
@@ -5432,7 +5406,7 @@
       <c r="I123" t="s">
         <v>307</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46296</v>
       </c>
       <c r="K123" t="b">
@@ -5467,7 +5441,7 @@
       <c r="I124" t="s">
         <v>308</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46293</v>
       </c>
       <c r="K124" t="b">
@@ -5502,7 +5476,7 @@
       <c r="I125" t="s">
         <v>309</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46305</v>
       </c>
       <c r="K125" t="b">
@@ -5534,7 +5508,7 @@
       <c r="H126">
         <v>-1476</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>43773</v>
       </c>
       <c r="K126" t="b">
@@ -5566,7 +5540,7 @@
       <c r="H127">
         <v>-1469</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>43773</v>
       </c>
       <c r="K127" t="b">
@@ -5598,7 +5572,7 @@
       <c r="H128">
         <v>-1250</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>45295</v>
       </c>
       <c r="K128" t="b">
@@ -5630,7 +5604,7 @@
       <c r="H129">
         <v>-1089</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>45617</v>
       </c>
       <c r="K129" t="b">
@@ -5662,7 +5636,7 @@
       <c r="H130">
         <v>-1021</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>45677</v>
       </c>
       <c r="K130" t="b">
@@ -5694,7 +5668,7 @@
       <c r="H131">
         <v>-1000</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>44944</v>
       </c>
       <c r="K131" t="b">
@@ -5726,7 +5700,7 @@
       <c r="H132">
         <v>-296</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46092</v>
       </c>
       <c r="K132" t="b">
@@ -5758,7 +5732,7 @@
       <c r="H133">
         <v>-51</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46258</v>
       </c>
       <c r="K133" t="b">
@@ -5790,7 +5764,7 @@
       <c r="H134">
         <v>-49</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46254</v>
       </c>
       <c r="K134" t="b">
@@ -5822,7 +5796,7 @@
       <c r="H135">
         <v>-49</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46254</v>
       </c>
       <c r="K135" t="b">
@@ -5854,7 +5828,7 @@
       <c r="H136">
         <v>43</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46440</v>
       </c>
       <c r="K136" t="b">
@@ -5886,7 +5860,7 @@
       <c r="H137">
         <v>43</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46440</v>
       </c>
       <c r="K137" t="b">
@@ -5918,7 +5892,7 @@
       <c r="H138">
         <v>102</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>46463</v>
       </c>
       <c r="K138" t="b">
@@ -5950,7 +5924,7 @@
       <c r="H139">
         <v>106</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>46424</v>
       </c>
       <c r="K139" t="b">
@@ -5982,7 +5956,7 @@
       <c r="H140">
         <v>119</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>46407</v>
       </c>
       <c r="K140" t="b">
@@ -6014,7 +5988,7 @@
       <c r="H141">
         <v>130</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>46416</v>
       </c>
       <c r="K141" t="b">
@@ -6046,7 +6020,7 @@
       <c r="H142">
         <v>152</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>46295</v>
       </c>
       <c r="K142" t="b">
@@ -6078,7 +6052,7 @@
       <c r="H143">
         <v>152</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46295</v>
       </c>
       <c r="K143" t="b">
@@ -6110,7 +6084,7 @@
       <c r="H144">
         <v>163</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46592</v>
       </c>
       <c r="K144" t="b">
@@ -6142,7 +6116,7 @@
       <c r="H145">
         <v>172</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46448</v>
       </c>
       <c r="K145" t="b">
@@ -6174,7 +6148,7 @@
       <c r="H146">
         <v>174</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46450</v>
       </c>
       <c r="K146" t="b">
@@ -6206,7 +6180,7 @@
       <c r="H147">
         <v>248</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46571</v>
       </c>
       <c r="K147" t="b">
@@ -6238,7 +6212,7 @@
       <c r="H148">
         <v>270</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46524</v>
       </c>
       <c r="K148" t="b">
@@ -6270,7 +6244,7 @@
       <c r="H149">
         <v>281</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46459</v>
       </c>
       <c r="K149" t="b">
@@ -6302,7 +6276,7 @@
       <c r="H150">
         <v>288</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46531</v>
       </c>
       <c r="K150" t="b">
@@ -6334,7 +6308,7 @@
       <c r="H151">
         <v>294</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46535</v>
       </c>
       <c r="K151" t="b">
@@ -6366,7 +6340,7 @@
       <c r="H152">
         <v>295</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46468</v>
       </c>
       <c r="K152" t="b">
@@ -6398,7 +6372,7 @@
       <c r="H153">
         <v>318</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46482</v>
       </c>
       <c r="K153" t="b">
@@ -6430,7 +6404,7 @@
       <c r="H154">
         <v>332</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46490</v>
       </c>
       <c r="K154" t="b">
@@ -6462,7 +6436,7 @@
       <c r="H155">
         <v>332</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46490</v>
       </c>
       <c r="K155" t="b">
@@ -6494,7 +6468,7 @@
       <c r="H156">
         <v>378</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46603</v>
       </c>
       <c r="K156" t="b">
@@ -6526,7 +6500,7 @@
       <c r="H157">
         <v>385</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46526</v>
       </c>
       <c r="K157" t="b">
@@ -6558,7 +6532,7 @@
       <c r="H158">
         <v>400</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46643</v>
       </c>
       <c r="K158" t="b">
@@ -6590,7 +6564,7 @@
       <c r="H159">
         <v>459</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46568</v>
       </c>
       <c r="K159" t="b">
@@ -6622,7 +6596,7 @@
       <c r="H160">
         <v>488</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46190</v>
       </c>
       <c r="K160" t="b">
@@ -6654,7 +6628,7 @@
       <c r="H161">
         <v>721</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46358</v>
       </c>
       <c r="K161" t="b">
@@ -6686,7 +6660,7 @@
       <c r="H162">
         <v>721</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46358</v>
       </c>
       <c r="K162" t="b">
@@ -6718,7 +6692,7 @@
       <c r="H163">
         <v>850</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46374</v>
       </c>
       <c r="K163" t="b">
@@ -6750,7 +6724,7 @@
       <c r="H164">
         <v>850</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46374</v>
       </c>
       <c r="K164" t="b">
@@ -6782,7 +6756,7 @@
       <c r="H165">
         <v>1661</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46529</v>
       </c>
       <c r="K165" t="b">
@@ -6814,7 +6788,7 @@
       <c r="H166">
         <v>1661</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46529</v>
       </c>
       <c r="K166" t="b">
@@ -6846,7 +6820,7 @@
       <c r="H167">
         <v>25565</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46190</v>
       </c>
       <c r="K167" t="b">
@@ -6878,7 +6852,7 @@
       <c r="H168">
         <v>25567</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46190</v>
       </c>
       <c r="K168" t="b">
@@ -6910,7 +6884,7 @@
       <c r="H169">
         <v>31293</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46190</v>
       </c>
       <c r="K169" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (13/10/2026 10:14)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3448,7 +3474,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3483,7 +3509,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3518,7 +3544,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3553,7 +3579,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3588,7 +3614,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3623,7 +3649,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3658,7 +3684,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3693,7 +3719,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3728,7 +3754,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3763,7 +3789,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3798,7 +3824,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3833,7 +3859,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3868,7 +3894,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3903,7 +3929,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3938,7 +3964,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3973,7 +3999,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4008,7 +4034,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4043,7 +4069,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4078,7 +4104,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4113,7 +4139,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4148,7 +4174,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4183,7 +4209,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4218,7 +4244,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4253,7 +4279,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4288,7 +4314,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4323,7 +4349,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4358,7 +4384,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4393,7 +4419,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4428,7 +4454,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4463,7 +4489,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4498,7 +4524,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4533,7 +4559,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4568,7 +4594,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4603,7 +4629,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4638,7 +4664,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4673,7 +4699,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4708,7 +4734,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4743,7 +4769,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4778,7 +4804,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4813,7 +4839,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4848,7 +4874,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4883,7 +4909,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4918,7 +4944,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4953,7 +4979,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -4988,7 +5014,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5023,7 +5049,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5058,7 +5084,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5093,7 +5119,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5128,7 +5154,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5163,7 +5189,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5198,7 +5224,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5233,7 +5259,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5268,7 +5294,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5303,7 +5329,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5338,7 +5364,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5373,7 +5399,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5408,7 +5434,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5443,7 +5469,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5478,7 +5504,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5513,7 +5539,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5548,7 +5574,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5583,7 +5609,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5618,7 +5644,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5653,7 +5679,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5688,7 +5714,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5723,7 +5749,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5758,7 +5784,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5793,7 +5819,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5828,7 +5854,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5863,7 +5889,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5898,7 +5924,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5933,7 +5959,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5968,7 +5994,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6000,7 +6026,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6032,7 +6058,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6064,7 +6090,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6096,7 +6122,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6128,7 +6154,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6160,7 +6186,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6192,7 +6218,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6224,7 +6250,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6256,7 +6282,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6288,7 +6314,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6320,7 +6346,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6352,7 +6378,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6384,7 +6410,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6416,7 +6442,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6448,7 +6474,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6480,7 +6506,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6512,7 +6538,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6544,7 +6570,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6576,7 +6602,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6608,7 +6634,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6640,7 +6666,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6672,7 +6698,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6704,7 +6730,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6736,7 +6762,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6768,7 +6794,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6800,7 +6826,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6832,7 +6858,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6864,7 +6890,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6896,7 +6922,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6928,7 +6954,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6960,7 +6986,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -6992,7 +7018,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7024,7 +7050,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7056,7 +7082,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7088,7 +7114,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7120,7 +7146,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7152,7 +7178,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7184,7 +7210,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7216,7 +7242,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7248,7 +7274,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7280,7 +7306,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7312,7 +7338,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7344,7 +7370,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7376,7 +7402,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7408,7 +7434,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7440,7 +7466,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7472,7 +7498,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (13/10/2026 15:08)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3474,7 +3448,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3509,7 +3483,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3544,7 +3518,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3579,7 +3553,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3614,7 +3588,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3649,7 +3623,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3684,7 +3658,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3719,7 +3693,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3754,7 +3728,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3789,7 +3763,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3824,7 +3798,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3859,7 +3833,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3894,7 +3868,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3929,7 +3903,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3964,7 +3938,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3999,7 +3973,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4034,7 +4008,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4069,7 +4043,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4104,7 +4078,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4139,7 +4113,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4174,7 +4148,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4209,7 +4183,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4244,7 +4218,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4279,7 +4253,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4314,7 +4288,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4349,7 +4323,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4384,7 +4358,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4419,7 +4393,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4454,7 +4428,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4489,7 +4463,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4524,7 +4498,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4559,7 +4533,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4594,7 +4568,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4629,7 +4603,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4664,7 +4638,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4699,7 +4673,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4734,7 +4708,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4769,7 +4743,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4804,7 +4778,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4839,7 +4813,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4874,7 +4848,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4909,7 +4883,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4944,7 +4918,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4979,7 +4953,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -5014,7 +4988,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5049,7 +5023,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5084,7 +5058,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5119,7 +5093,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5154,7 +5128,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5189,7 +5163,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5224,7 +5198,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5259,7 +5233,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5294,7 +5268,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5329,7 +5303,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5364,7 +5338,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5399,7 +5373,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5434,7 +5408,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5469,7 +5443,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5504,7 +5478,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5539,7 +5513,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5574,7 +5548,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5609,7 +5583,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5644,7 +5618,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5679,7 +5653,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5714,7 +5688,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5749,7 +5723,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5784,7 +5758,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5819,7 +5793,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5854,7 +5828,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5889,7 +5863,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5924,7 +5898,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5959,7 +5933,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5994,7 +5968,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6026,7 +6000,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6058,7 +6032,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6090,7 +6064,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6122,7 +6096,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6154,7 +6128,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6186,7 +6160,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6218,7 +6192,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6250,7 +6224,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6282,7 +6256,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6314,7 +6288,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6346,7 +6320,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6378,7 +6352,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6410,7 +6384,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6442,7 +6416,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6474,7 +6448,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6506,7 +6480,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6538,7 +6512,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6570,7 +6544,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6602,7 +6576,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6634,7 +6608,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6666,7 +6640,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6698,7 +6672,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6730,7 +6704,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6762,7 +6736,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6794,7 +6768,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6826,7 +6800,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6858,7 +6832,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6890,7 +6864,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6922,7 +6896,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6954,7 +6928,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6986,7 +6960,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -7018,7 +6992,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7050,7 +7024,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7082,7 +7056,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7114,7 +7088,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7146,7 +7120,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7178,7 +7152,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7210,7 +7184,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7242,7 +7216,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7274,7 +7248,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7306,7 +7280,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7338,7 +7312,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7370,7 +7344,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7402,7 +7376,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7434,7 +7408,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7466,7 +7440,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7498,7 +7472,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (14/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3448,7 +3474,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3483,7 +3509,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3518,7 +3544,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3553,7 +3579,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3588,7 +3614,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3623,7 +3649,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3658,7 +3684,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3693,7 +3719,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3728,7 +3754,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3763,7 +3789,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3798,7 +3824,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3833,7 +3859,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3868,7 +3894,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3903,7 +3929,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3938,7 +3964,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3973,7 +3999,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4008,7 +4034,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4043,7 +4069,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4078,7 +4104,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4113,7 +4139,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4148,7 +4174,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4183,7 +4209,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4218,7 +4244,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4253,7 +4279,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4288,7 +4314,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4323,7 +4349,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4358,7 +4384,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4393,7 +4419,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4428,7 +4454,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4463,7 +4489,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4498,7 +4524,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4533,7 +4559,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4568,7 +4594,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4603,7 +4629,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4638,7 +4664,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4673,7 +4699,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4708,7 +4734,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4743,7 +4769,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4778,7 +4804,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4813,7 +4839,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4848,7 +4874,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4883,7 +4909,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4918,7 +4944,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4953,7 +4979,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -4988,7 +5014,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5023,7 +5049,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5058,7 +5084,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5093,7 +5119,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5128,7 +5154,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5163,7 +5189,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5198,7 +5224,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5233,7 +5259,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5268,7 +5294,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5303,7 +5329,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5338,7 +5364,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5373,7 +5399,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5408,7 +5434,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5443,7 +5469,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5478,7 +5504,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5513,7 +5539,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5548,7 +5574,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5583,7 +5609,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5618,7 +5644,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5653,7 +5679,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5688,7 +5714,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5723,7 +5749,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5758,7 +5784,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5793,7 +5819,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5828,7 +5854,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5863,7 +5889,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5898,7 +5924,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5933,7 +5959,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5968,7 +5994,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6000,7 +6026,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6032,7 +6058,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6064,7 +6090,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6096,7 +6122,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6128,7 +6154,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6160,7 +6186,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6192,7 +6218,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6224,7 +6250,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6256,7 +6282,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6288,7 +6314,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6320,7 +6346,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6352,7 +6378,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6384,7 +6410,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6416,7 +6442,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6448,7 +6474,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6480,7 +6506,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6512,7 +6538,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6544,7 +6570,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6576,7 +6602,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6608,7 +6634,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6640,7 +6666,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6672,7 +6698,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6704,7 +6730,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6736,7 +6762,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6768,7 +6794,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6800,7 +6826,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6832,7 +6858,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6864,7 +6890,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6896,7 +6922,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6928,7 +6954,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6960,7 +6986,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -6992,7 +7018,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7024,7 +7050,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7056,7 +7082,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7088,7 +7114,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7120,7 +7146,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7152,7 +7178,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7184,7 +7210,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7216,7 +7242,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7248,7 +7274,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7280,7 +7306,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7312,7 +7338,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7344,7 +7370,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7376,7 +7402,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7408,7 +7434,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7440,7 +7466,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7472,7 +7498,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (15/10/2026 12:34)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3474,7 +3448,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3509,7 +3483,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3544,7 +3518,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3579,7 +3553,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3614,7 +3588,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3649,7 +3623,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3684,7 +3658,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3719,7 +3693,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3754,7 +3728,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3789,7 +3763,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3824,7 +3798,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3859,7 +3833,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3894,7 +3868,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3929,7 +3903,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3964,7 +3938,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3999,7 +3973,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4034,7 +4008,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4069,7 +4043,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4104,7 +4078,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4139,7 +4113,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4174,7 +4148,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4209,7 +4183,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4244,7 +4218,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4279,7 +4253,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4314,7 +4288,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4349,7 +4323,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4384,7 +4358,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4419,7 +4393,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4454,7 +4428,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4489,7 +4463,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4524,7 +4498,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4559,7 +4533,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4594,7 +4568,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4629,7 +4603,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4664,7 +4638,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4699,7 +4673,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4734,7 +4708,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4769,7 +4743,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4804,7 +4778,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4839,7 +4813,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4874,7 +4848,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4909,7 +4883,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4944,7 +4918,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4979,7 +4953,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -5014,7 +4988,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5049,7 +5023,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5084,7 +5058,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5119,7 +5093,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5154,7 +5128,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5189,7 +5163,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5224,7 +5198,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5259,7 +5233,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5294,7 +5268,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5329,7 +5303,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5364,7 +5338,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5399,7 +5373,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5434,7 +5408,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5469,7 +5443,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5504,7 +5478,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5539,7 +5513,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5574,7 +5548,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5609,7 +5583,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5644,7 +5618,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5679,7 +5653,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5714,7 +5688,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5749,7 +5723,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5784,7 +5758,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5819,7 +5793,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5854,7 +5828,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5889,7 +5863,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5924,7 +5898,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5959,7 +5933,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5994,7 +5968,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6026,7 +6000,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6058,7 +6032,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6090,7 +6064,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6122,7 +6096,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6154,7 +6128,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6186,7 +6160,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6218,7 +6192,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6250,7 +6224,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6282,7 +6256,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6314,7 +6288,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6346,7 +6320,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6378,7 +6352,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6410,7 +6384,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6442,7 +6416,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6474,7 +6448,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6506,7 +6480,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6538,7 +6512,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6570,7 +6544,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6602,7 +6576,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6634,7 +6608,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6666,7 +6640,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6698,7 +6672,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6730,7 +6704,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6762,7 +6736,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6794,7 +6768,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6826,7 +6800,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6858,7 +6832,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6890,7 +6864,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6922,7 +6896,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6954,7 +6928,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6986,7 +6960,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -7018,7 +6992,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7050,7 +7024,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7082,7 +7056,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7114,7 +7088,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7146,7 +7120,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7178,7 +7152,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7210,7 +7184,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7242,7 +7216,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7274,7 +7248,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7306,7 +7280,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7338,7 +7312,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7370,7 +7344,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7402,7 +7376,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7434,7 +7408,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7466,7 +7440,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7498,7 +7472,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (16/10/2026 12:02)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3448,7 +3474,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3483,7 +3509,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3518,7 +3544,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3553,7 +3579,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3588,7 +3614,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3623,7 +3649,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3658,7 +3684,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3693,7 +3719,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3728,7 +3754,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3763,7 +3789,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3798,7 +3824,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3833,7 +3859,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3868,7 +3894,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3903,7 +3929,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3938,7 +3964,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3973,7 +3999,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4008,7 +4034,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4043,7 +4069,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4078,7 +4104,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4113,7 +4139,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4148,7 +4174,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4183,7 +4209,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4218,7 +4244,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4253,7 +4279,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4288,7 +4314,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4323,7 +4349,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4358,7 +4384,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4393,7 +4419,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4428,7 +4454,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4463,7 +4489,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4498,7 +4524,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4533,7 +4559,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4568,7 +4594,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4603,7 +4629,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4638,7 +4664,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4673,7 +4699,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4708,7 +4734,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4743,7 +4769,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4778,7 +4804,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4813,7 +4839,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4848,7 +4874,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4883,7 +4909,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4918,7 +4944,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4953,7 +4979,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -4988,7 +5014,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5023,7 +5049,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5058,7 +5084,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5093,7 +5119,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5128,7 +5154,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5163,7 +5189,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5198,7 +5224,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5233,7 +5259,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5268,7 +5294,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5303,7 +5329,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5338,7 +5364,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5373,7 +5399,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5408,7 +5434,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5443,7 +5469,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5478,7 +5504,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5513,7 +5539,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5548,7 +5574,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5583,7 +5609,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5618,7 +5644,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5653,7 +5679,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5688,7 +5714,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5723,7 +5749,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5758,7 +5784,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5793,7 +5819,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5828,7 +5854,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5863,7 +5889,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5898,7 +5924,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5933,7 +5959,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5968,7 +5994,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6000,7 +6026,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6032,7 +6058,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6064,7 +6090,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6096,7 +6122,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6128,7 +6154,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6160,7 +6186,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6192,7 +6218,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6224,7 +6250,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6256,7 +6282,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6288,7 +6314,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6320,7 +6346,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6352,7 +6378,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6384,7 +6410,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6416,7 +6442,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6448,7 +6474,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6480,7 +6506,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6512,7 +6538,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6544,7 +6570,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6576,7 +6602,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6608,7 +6634,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6640,7 +6666,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6672,7 +6698,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6704,7 +6730,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6736,7 +6762,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6768,7 +6794,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6800,7 +6826,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6832,7 +6858,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6864,7 +6890,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6896,7 +6922,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6928,7 +6954,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6960,7 +6986,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -6992,7 +7018,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7024,7 +7050,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7056,7 +7082,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7088,7 +7114,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7120,7 +7146,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7152,7 +7178,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7184,7 +7210,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7216,7 +7242,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7248,7 +7274,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7280,7 +7306,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7312,7 +7338,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7344,7 +7370,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7376,7 +7402,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7408,7 +7434,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7440,7 +7466,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7472,7 +7498,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (16/10/2026 12:21)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3474,7 +3448,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3509,7 +3483,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3544,7 +3518,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3579,7 +3553,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3614,7 +3588,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3649,7 +3623,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3684,7 +3658,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3719,7 +3693,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3754,7 +3728,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3789,7 +3763,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3824,7 +3798,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3859,7 +3833,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3894,7 +3868,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3929,7 +3903,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3964,7 +3938,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3999,7 +3973,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4034,7 +4008,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4069,7 +4043,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4104,7 +4078,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4139,7 +4113,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4174,7 +4148,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4209,7 +4183,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4244,7 +4218,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4279,7 +4253,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4314,7 +4288,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4349,7 +4323,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4384,7 +4358,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4419,7 +4393,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4454,7 +4428,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4489,7 +4463,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4524,7 +4498,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4559,7 +4533,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4594,7 +4568,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4629,7 +4603,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4664,7 +4638,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4699,7 +4673,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4734,7 +4708,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4769,7 +4743,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4804,7 +4778,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4839,7 +4813,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4874,7 +4848,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4909,7 +4883,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4944,7 +4918,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4979,7 +4953,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -5014,7 +4988,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5049,7 +5023,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5084,7 +5058,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5119,7 +5093,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5154,7 +5128,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5189,7 +5163,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5224,7 +5198,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5259,7 +5233,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5294,7 +5268,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5329,7 +5303,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5364,7 +5338,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5399,7 +5373,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5434,7 +5408,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5469,7 +5443,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5504,7 +5478,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5539,7 +5513,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5574,7 +5548,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5609,7 +5583,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5644,7 +5618,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5679,7 +5653,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5714,7 +5688,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5749,7 +5723,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5784,7 +5758,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5819,7 +5793,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5854,7 +5828,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5889,7 +5863,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5924,7 +5898,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5959,7 +5933,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5994,7 +5968,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6026,7 +6000,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6058,7 +6032,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6090,7 +6064,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6122,7 +6096,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6154,7 +6128,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6186,7 +6160,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6218,7 +6192,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6250,7 +6224,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6282,7 +6256,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6314,7 +6288,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6346,7 +6320,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6378,7 +6352,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6410,7 +6384,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6442,7 +6416,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6474,7 +6448,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6506,7 +6480,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6538,7 +6512,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6570,7 +6544,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6602,7 +6576,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6634,7 +6608,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6666,7 +6640,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6698,7 +6672,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6730,7 +6704,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6762,7 +6736,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6794,7 +6768,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6826,7 +6800,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6858,7 +6832,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6890,7 +6864,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6922,7 +6896,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6954,7 +6928,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6986,7 +6960,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -7018,7 +6992,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7050,7 +7024,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7082,7 +7056,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7114,7 +7088,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7146,7 +7120,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7178,7 +7152,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7210,7 +7184,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7242,7 +7216,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7274,7 +7248,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7306,7 +7280,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7338,7 +7312,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7370,7 +7344,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7402,7 +7376,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7434,7 +7408,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7466,7 +7440,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7498,7 +7472,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (19/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3448,7 +3474,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3483,7 +3509,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3518,7 +3544,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3553,7 +3579,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3588,7 +3614,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3623,7 +3649,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3658,7 +3684,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3693,7 +3719,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3728,7 +3754,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3763,7 +3789,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3798,7 +3824,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3833,7 +3859,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3868,7 +3894,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3903,7 +3929,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3938,7 +3964,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3973,7 +3999,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4008,7 +4034,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4043,7 +4069,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4078,7 +4104,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4113,7 +4139,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4148,7 +4174,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4183,7 +4209,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4218,7 +4244,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4253,7 +4279,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4288,7 +4314,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4323,7 +4349,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4358,7 +4384,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4393,7 +4419,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4428,7 +4454,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4463,7 +4489,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4498,7 +4524,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4533,7 +4559,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4568,7 +4594,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4603,7 +4629,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4638,7 +4664,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4673,7 +4699,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4708,7 +4734,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4743,7 +4769,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4778,7 +4804,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4813,7 +4839,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4848,7 +4874,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4883,7 +4909,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4918,7 +4944,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4953,7 +4979,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -4988,7 +5014,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5023,7 +5049,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5058,7 +5084,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5093,7 +5119,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5128,7 +5154,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5163,7 +5189,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5198,7 +5224,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5233,7 +5259,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5268,7 +5294,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5303,7 +5329,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5338,7 +5364,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5373,7 +5399,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5408,7 +5434,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5443,7 +5469,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5478,7 +5504,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5513,7 +5539,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5548,7 +5574,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5583,7 +5609,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5618,7 +5644,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5653,7 +5679,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5688,7 +5714,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5723,7 +5749,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5758,7 +5784,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5793,7 +5819,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5828,7 +5854,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5863,7 +5889,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5898,7 +5924,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5933,7 +5959,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5968,7 +5994,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6000,7 +6026,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6032,7 +6058,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6064,7 +6090,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6096,7 +6122,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6128,7 +6154,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6160,7 +6186,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6192,7 +6218,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6224,7 +6250,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6256,7 +6282,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6288,7 +6314,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6320,7 +6346,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6352,7 +6378,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6384,7 +6410,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6416,7 +6442,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6448,7 +6474,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6480,7 +6506,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6512,7 +6538,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6544,7 +6570,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6576,7 +6602,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6608,7 +6634,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6640,7 +6666,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6672,7 +6698,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6704,7 +6730,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6736,7 +6762,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6768,7 +6794,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6800,7 +6826,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6832,7 +6858,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6864,7 +6890,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6896,7 +6922,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6928,7 +6954,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6960,7 +6986,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -6992,7 +7018,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7024,7 +7050,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7056,7 +7082,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7088,7 +7114,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7120,7 +7146,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7152,7 +7178,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7184,7 +7210,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7216,7 +7242,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7248,7 +7274,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7280,7 +7306,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7312,7 +7338,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7344,7 +7370,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7376,7 +7402,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7408,7 +7434,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7440,7 +7466,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7472,7 +7498,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (19/10/2026 14:26)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3474,7 +3448,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3509,7 +3483,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3544,7 +3518,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3579,7 +3553,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3614,7 +3588,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3649,7 +3623,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3684,7 +3658,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3719,7 +3693,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3754,7 +3728,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3789,7 +3763,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3824,7 +3798,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3859,7 +3833,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3894,7 +3868,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3929,7 +3903,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3964,7 +3938,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3999,7 +3973,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4034,7 +4008,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4069,7 +4043,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4104,7 +4078,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4139,7 +4113,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4174,7 +4148,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4209,7 +4183,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4244,7 +4218,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4279,7 +4253,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4314,7 +4288,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4349,7 +4323,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4384,7 +4358,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4419,7 +4393,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4454,7 +4428,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4489,7 +4463,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4524,7 +4498,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4559,7 +4533,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4594,7 +4568,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4629,7 +4603,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4664,7 +4638,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4699,7 +4673,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4734,7 +4708,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4769,7 +4743,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4804,7 +4778,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4839,7 +4813,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4874,7 +4848,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4909,7 +4883,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4944,7 +4918,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4979,7 +4953,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -5014,7 +4988,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5049,7 +5023,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5084,7 +5058,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5119,7 +5093,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5154,7 +5128,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5189,7 +5163,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5224,7 +5198,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5259,7 +5233,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5294,7 +5268,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5329,7 +5303,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5364,7 +5338,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5399,7 +5373,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5434,7 +5408,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5469,7 +5443,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5504,7 +5478,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5539,7 +5513,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5574,7 +5548,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5609,7 +5583,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5644,7 +5618,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5679,7 +5653,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5714,7 +5688,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5749,7 +5723,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5784,7 +5758,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5819,7 +5793,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5854,7 +5828,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5889,7 +5863,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5924,7 +5898,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5959,7 +5933,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5994,7 +5968,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6026,7 +6000,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6058,7 +6032,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6090,7 +6064,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6122,7 +6096,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6154,7 +6128,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6186,7 +6160,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6218,7 +6192,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6250,7 +6224,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6282,7 +6256,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6314,7 +6288,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6346,7 +6320,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6378,7 +6352,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6410,7 +6384,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6442,7 +6416,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6474,7 +6448,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6506,7 +6480,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6538,7 +6512,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6570,7 +6544,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6602,7 +6576,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6634,7 +6608,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6666,7 +6640,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6698,7 +6672,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6730,7 +6704,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6762,7 +6736,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6794,7 +6768,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6826,7 +6800,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6858,7 +6832,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6890,7 +6864,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6922,7 +6896,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6954,7 +6928,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6986,7 +6960,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -7018,7 +6992,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7050,7 +7024,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7082,7 +7056,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7114,7 +7088,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7146,7 +7120,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7178,7 +7152,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7210,7 +7184,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7242,7 +7216,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7274,7 +7248,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7306,7 +7280,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7338,7 +7312,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7370,7 +7344,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7402,7 +7376,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7434,7 +7408,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7466,7 +7440,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7498,7 +7472,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (20/10/2026 12:03)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3448,7 +3474,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3483,7 +3509,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3518,7 +3544,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3553,7 +3579,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3588,7 +3614,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3623,7 +3649,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3658,7 +3684,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3693,7 +3719,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3728,7 +3754,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3763,7 +3789,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3798,7 +3824,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3833,7 +3859,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3868,7 +3894,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3903,7 +3929,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3938,7 +3964,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3973,7 +3999,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4008,7 +4034,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4043,7 +4069,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4078,7 +4104,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4113,7 +4139,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4148,7 +4174,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4183,7 +4209,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4218,7 +4244,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4253,7 +4279,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4288,7 +4314,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4323,7 +4349,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4358,7 +4384,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4393,7 +4419,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4428,7 +4454,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4463,7 +4489,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4498,7 +4524,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4533,7 +4559,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4568,7 +4594,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4603,7 +4629,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4638,7 +4664,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4673,7 +4699,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4708,7 +4734,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4743,7 +4769,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4778,7 +4804,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4813,7 +4839,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4848,7 +4874,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4883,7 +4909,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4918,7 +4944,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4953,7 +4979,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -4988,7 +5014,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5023,7 +5049,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5058,7 +5084,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5093,7 +5119,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5128,7 +5154,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5163,7 +5189,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5198,7 +5224,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5233,7 +5259,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5268,7 +5294,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5303,7 +5329,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5338,7 +5364,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5373,7 +5399,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5408,7 +5434,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5443,7 +5469,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5478,7 +5504,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5513,7 +5539,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5548,7 +5574,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5583,7 +5609,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5618,7 +5644,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5653,7 +5679,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5688,7 +5714,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5723,7 +5749,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5758,7 +5784,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5793,7 +5819,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5828,7 +5854,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5863,7 +5889,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5898,7 +5924,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5933,7 +5959,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5968,7 +5994,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6000,7 +6026,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6032,7 +6058,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6064,7 +6090,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6096,7 +6122,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6128,7 +6154,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6160,7 +6186,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6192,7 +6218,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6224,7 +6250,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6256,7 +6282,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6288,7 +6314,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6320,7 +6346,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6352,7 +6378,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6384,7 +6410,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6416,7 +6442,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6448,7 +6474,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6480,7 +6506,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6512,7 +6538,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6544,7 +6570,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6576,7 +6602,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6608,7 +6634,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6640,7 +6666,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6672,7 +6698,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6704,7 +6730,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6736,7 +6762,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6768,7 +6794,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6800,7 +6826,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6832,7 +6858,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6864,7 +6890,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6896,7 +6922,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6928,7 +6954,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6960,7 +6986,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -6992,7 +7018,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7024,7 +7050,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7056,7 +7082,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7088,7 +7114,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7120,7 +7146,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7152,7 +7178,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7184,7 +7210,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7216,7 +7242,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7248,7 +7274,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7280,7 +7306,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7312,7 +7338,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7344,7 +7370,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7376,7 +7402,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7408,7 +7434,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7440,7 +7466,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7472,7 +7498,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (20/10/2026 12:38)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3474,7 +3448,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3509,7 +3483,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3544,7 +3518,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3579,7 +3553,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3614,7 +3588,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3649,7 +3623,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3684,7 +3658,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3719,7 +3693,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3754,7 +3728,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3789,7 +3763,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3824,7 +3798,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3859,7 +3833,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3894,7 +3868,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3929,7 +3903,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3964,7 +3938,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3999,7 +3973,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4034,7 +4008,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4069,7 +4043,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4104,7 +4078,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4139,7 +4113,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4174,7 +4148,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4209,7 +4183,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4244,7 +4218,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4279,7 +4253,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4314,7 +4288,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4349,7 +4323,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4384,7 +4358,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4419,7 +4393,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4454,7 +4428,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4489,7 +4463,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4524,7 +4498,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4559,7 +4533,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4594,7 +4568,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4629,7 +4603,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4664,7 +4638,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4699,7 +4673,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4734,7 +4708,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4769,7 +4743,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4804,7 +4778,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4839,7 +4813,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4874,7 +4848,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4909,7 +4883,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4944,7 +4918,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4979,7 +4953,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -5014,7 +4988,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5049,7 +5023,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5084,7 +5058,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5119,7 +5093,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5154,7 +5128,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5189,7 +5163,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5224,7 +5198,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5259,7 +5233,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5294,7 +5268,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5329,7 +5303,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5364,7 +5338,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5399,7 +5373,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5434,7 +5408,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5469,7 +5443,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5504,7 +5478,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5539,7 +5513,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5574,7 +5548,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5609,7 +5583,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5644,7 +5618,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5679,7 +5653,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5714,7 +5688,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5749,7 +5723,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5784,7 +5758,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5819,7 +5793,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5854,7 +5828,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5889,7 +5863,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5924,7 +5898,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5959,7 +5933,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5994,7 +5968,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6026,7 +6000,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6058,7 +6032,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6090,7 +6064,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6122,7 +6096,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6154,7 +6128,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6186,7 +6160,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6218,7 +6192,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6250,7 +6224,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6282,7 +6256,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6314,7 +6288,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6346,7 +6320,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6378,7 +6352,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6410,7 +6384,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6442,7 +6416,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6474,7 +6448,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6506,7 +6480,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6538,7 +6512,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6570,7 +6544,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6602,7 +6576,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6634,7 +6608,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6666,7 +6640,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6698,7 +6672,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6730,7 +6704,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6762,7 +6736,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6794,7 +6768,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6826,7 +6800,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6858,7 +6832,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6890,7 +6864,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6922,7 +6896,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6954,7 +6928,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6986,7 +6960,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -7018,7 +6992,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7050,7 +7024,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7082,7 +7056,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7114,7 +7088,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7146,7 +7120,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7178,7 +7152,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7210,7 +7184,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7242,7 +7216,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7274,7 +7248,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7306,7 +7280,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7338,7 +7312,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7370,7 +7344,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7402,7 +7376,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7434,7 +7408,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7466,7 +7440,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7498,7 +7472,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (21/10/2026 14:22)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3448,7 +3474,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3483,7 +3509,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3518,7 +3544,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3553,7 +3579,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3588,7 +3614,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3623,7 +3649,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3658,7 +3684,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3693,7 +3719,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3728,7 +3754,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3763,7 +3789,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3798,7 +3824,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3833,7 +3859,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3868,7 +3894,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3903,7 +3929,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3938,7 +3964,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3973,7 +3999,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4008,7 +4034,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4043,7 +4069,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4078,7 +4104,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4113,7 +4139,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4148,7 +4174,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4183,7 +4209,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4218,7 +4244,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4253,7 +4279,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4288,7 +4314,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4323,7 +4349,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4358,7 +4384,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4393,7 +4419,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4428,7 +4454,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4463,7 +4489,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4498,7 +4524,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4533,7 +4559,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4568,7 +4594,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4603,7 +4629,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4638,7 +4664,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4673,7 +4699,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4708,7 +4734,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4743,7 +4769,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4778,7 +4804,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4813,7 +4839,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4848,7 +4874,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4883,7 +4909,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4918,7 +4944,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4953,7 +4979,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -4988,7 +5014,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5023,7 +5049,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5058,7 +5084,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5093,7 +5119,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5128,7 +5154,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5163,7 +5189,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5198,7 +5224,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5233,7 +5259,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5268,7 +5294,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5303,7 +5329,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5338,7 +5364,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5373,7 +5399,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5408,7 +5434,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5443,7 +5469,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5478,7 +5504,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5513,7 +5539,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5548,7 +5574,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5583,7 +5609,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5618,7 +5644,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5653,7 +5679,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5688,7 +5714,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5723,7 +5749,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5758,7 +5784,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5793,7 +5819,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5828,7 +5854,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5863,7 +5889,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5898,7 +5924,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5933,7 +5959,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5968,7 +5994,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6000,7 +6026,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6032,7 +6058,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6064,7 +6090,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6096,7 +6122,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6128,7 +6154,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6160,7 +6186,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6192,7 +6218,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6224,7 +6250,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6256,7 +6282,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6288,7 +6314,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6320,7 +6346,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6352,7 +6378,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6384,7 +6410,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6416,7 +6442,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6448,7 +6474,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6480,7 +6506,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6512,7 +6538,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6544,7 +6570,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6576,7 +6602,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6608,7 +6634,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6640,7 +6666,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6672,7 +6698,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6704,7 +6730,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6736,7 +6762,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6768,7 +6794,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6800,7 +6826,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6832,7 +6858,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6864,7 +6890,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6896,7 +6922,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6928,7 +6954,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6960,7 +6986,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -6992,7 +7018,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7024,7 +7050,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7056,7 +7082,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7088,7 +7114,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7120,7 +7146,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7152,7 +7178,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7184,7 +7210,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7216,7 +7242,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7248,7 +7274,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7280,7 +7306,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7312,7 +7338,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7344,7 +7370,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7376,7 +7402,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7408,7 +7434,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7440,7 +7466,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7472,7 +7498,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (22/10/2026 12:52)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3474,7 +3448,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3509,7 +3483,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3544,7 +3518,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3579,7 +3553,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3614,7 +3588,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3649,7 +3623,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3684,7 +3658,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3719,7 +3693,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3754,7 +3728,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3789,7 +3763,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3824,7 +3798,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3859,7 +3833,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3894,7 +3868,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3929,7 +3903,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3964,7 +3938,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3999,7 +3973,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4034,7 +4008,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4069,7 +4043,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4104,7 +4078,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4139,7 +4113,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4174,7 +4148,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4209,7 +4183,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4244,7 +4218,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4279,7 +4253,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4314,7 +4288,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4349,7 +4323,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4384,7 +4358,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4419,7 +4393,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4454,7 +4428,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4489,7 +4463,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4524,7 +4498,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4559,7 +4533,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4594,7 +4568,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4629,7 +4603,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4664,7 +4638,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4699,7 +4673,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4734,7 +4708,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4769,7 +4743,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4804,7 +4778,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4839,7 +4813,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4874,7 +4848,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4909,7 +4883,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4944,7 +4918,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4979,7 +4953,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -5014,7 +4988,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5049,7 +5023,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5084,7 +5058,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5119,7 +5093,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5154,7 +5128,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5189,7 +5163,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5224,7 +5198,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5259,7 +5233,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5294,7 +5268,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5329,7 +5303,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5364,7 +5338,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5399,7 +5373,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5434,7 +5408,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5469,7 +5443,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5504,7 +5478,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5539,7 +5513,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5574,7 +5548,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5609,7 +5583,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5644,7 +5618,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5679,7 +5653,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5714,7 +5688,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5749,7 +5723,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5784,7 +5758,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5819,7 +5793,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5854,7 +5828,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5889,7 +5863,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5924,7 +5898,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5959,7 +5933,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5994,7 +5968,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6026,7 +6000,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6058,7 +6032,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6090,7 +6064,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6122,7 +6096,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6154,7 +6128,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6186,7 +6160,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6218,7 +6192,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6250,7 +6224,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6282,7 +6256,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6314,7 +6288,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6346,7 +6320,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6378,7 +6352,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6410,7 +6384,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6442,7 +6416,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6474,7 +6448,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6506,7 +6480,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6538,7 +6512,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6570,7 +6544,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6602,7 +6576,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6634,7 +6608,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6666,7 +6640,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6698,7 +6672,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6730,7 +6704,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6762,7 +6736,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6794,7 +6768,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6826,7 +6800,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6858,7 +6832,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6890,7 +6864,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6922,7 +6896,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6954,7 +6928,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6986,7 +6960,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -7018,7 +6992,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7050,7 +7024,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7082,7 +7056,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7114,7 +7088,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7146,7 +7120,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7178,7 +7152,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7210,7 +7184,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7242,7 +7216,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7274,7 +7248,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7306,7 +7280,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7338,7 +7312,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7370,7 +7344,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7402,7 +7376,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7434,7 +7408,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7466,7 +7440,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7498,7 +7472,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (23/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,8 +1040,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1057,7 +1065,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1065,12 +1073,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1370,37 +1396,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1429,7 +1455,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1461,7 +1487,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1493,7 +1519,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1525,7 +1551,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1557,7 +1583,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1589,7 +1615,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1621,7 +1647,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1653,7 +1679,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1685,7 +1711,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1717,7 +1743,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1749,7 +1775,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1781,7 +1807,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1813,7 +1839,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1845,7 +1871,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1877,7 +1903,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1909,7 +1935,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1941,7 +1967,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1973,7 +1999,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2005,7 +2031,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2037,7 +2063,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2069,7 +2095,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2101,7 +2127,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2133,7 +2159,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2165,7 +2191,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2197,7 +2223,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2229,7 +2255,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2261,7 +2287,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="1">
+      <c r="J28" s="2">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2293,7 +2319,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="1">
+      <c r="J29" s="2">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2325,7 +2351,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="1">
+      <c r="J30" s="2">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2357,7 +2383,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="1">
+      <c r="J31" s="2">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2389,7 +2415,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="1">
+      <c r="J32" s="2">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2421,7 +2447,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="1">
+      <c r="J33" s="2">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2453,7 +2479,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="1">
+      <c r="J34" s="2">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2485,7 +2511,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="1">
+      <c r="J35" s="2">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2517,7 +2543,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="1">
+      <c r="J36" s="2">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2549,7 +2575,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="1">
+      <c r="J37" s="2">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2581,7 +2607,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="1">
+      <c r="J38" s="2">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2613,7 +2639,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="1">
+      <c r="J39" s="2">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2645,7 +2671,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="1">
+      <c r="J40" s="2">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2677,7 +2703,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="J41" s="2">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2709,7 +2735,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="2">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2741,7 +2767,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="1">
+      <c r="J43" s="2">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2773,7 +2799,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="1">
+      <c r="J44" s="2">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2805,7 +2831,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="1">
+      <c r="J45" s="2">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2837,7 +2863,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="2">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2869,7 +2895,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="1">
+      <c r="J47" s="2">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2901,7 +2927,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="1">
+      <c r="J48" s="2">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2933,7 +2959,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="1">
+      <c r="J49" s="2">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2965,7 +2991,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="1">
+      <c r="J50" s="2">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -2997,7 +3023,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="1">
+      <c r="J51" s="2">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3029,7 +3055,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="1">
+      <c r="J52" s="2">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3061,7 +3087,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="1">
+      <c r="J53" s="2">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3093,7 +3119,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="1">
+      <c r="J54" s="2">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3125,7 +3151,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="1">
+      <c r="J55" s="2">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3157,7 +3183,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="1">
+      <c r="J56" s="2">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3189,7 +3215,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="1">
+      <c r="J57" s="2">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3221,7 +3247,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="1">
+      <c r="J58" s="2">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3253,7 +3279,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="1">
+      <c r="J59" s="2">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3285,7 +3311,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="1">
+      <c r="J60" s="2">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3317,7 +3343,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="1">
+      <c r="J61" s="2">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3349,7 +3375,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="1">
+      <c r="J62" s="2">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3381,7 +3407,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="1">
+      <c r="J63" s="2">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3413,7 +3439,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="1">
+      <c r="J64" s="2">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3448,7 +3474,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="1">
+      <c r="J65" s="2">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3483,7 +3509,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="1">
+      <c r="J66" s="2">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3518,7 +3544,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="1">
+      <c r="J67" s="2">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3553,7 +3579,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="1">
+      <c r="J68" s="2">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3588,7 +3614,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="1">
+      <c r="J69" s="2">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3623,7 +3649,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="1">
+      <c r="J70" s="2">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3658,7 +3684,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="1">
+      <c r="J71" s="2">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3693,7 +3719,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="1">
+      <c r="J72" s="2">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3728,7 +3754,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="1">
+      <c r="J73" s="2">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3763,7 +3789,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="1">
+      <c r="J74" s="2">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3798,7 +3824,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="1">
+      <c r="J75" s="2">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3833,7 +3859,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="1">
+      <c r="J76" s="2">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3868,7 +3894,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="1">
+      <c r="J77" s="2">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3903,7 +3929,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="1">
+      <c r="J78" s="2">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3938,7 +3964,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="1">
+      <c r="J79" s="2">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3973,7 +3999,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="1">
+      <c r="J80" s="2">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4008,7 +4034,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="1">
+      <c r="J81" s="2">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4043,7 +4069,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="1">
+      <c r="J82" s="2">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4078,7 +4104,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="1">
+      <c r="J83" s="2">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4113,7 +4139,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="1">
+      <c r="J84" s="2">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4148,7 +4174,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="1">
+      <c r="J85" s="2">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4183,7 +4209,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="1">
+      <c r="J86" s="2">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4218,7 +4244,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="1">
+      <c r="J87" s="2">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4253,7 +4279,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="1">
+      <c r="J88" s="2">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4288,7 +4314,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="1">
+      <c r="J89" s="2">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4323,7 +4349,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="1">
+      <c r="J90" s="2">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4358,7 +4384,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="1">
+      <c r="J91" s="2">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4393,7 +4419,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="1">
+      <c r="J92" s="2">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4428,7 +4454,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="1">
+      <c r="J93" s="2">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4463,7 +4489,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="1">
+      <c r="J94" s="2">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4498,7 +4524,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="1">
+      <c r="J95" s="2">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4533,7 +4559,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="1">
+      <c r="J96" s="2">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4568,7 +4594,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="1">
+      <c r="J97" s="2">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4603,7 +4629,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="1">
+      <c r="J98" s="2">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4638,7 +4664,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="1">
+      <c r="J99" s="2">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4673,7 +4699,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="1">
+      <c r="J100" s="2">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4708,7 +4734,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="1">
+      <c r="J101" s="2">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4743,7 +4769,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="1">
+      <c r="J102" s="2">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4778,7 +4804,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="1">
+      <c r="J103" s="2">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4813,7 +4839,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="1">
+      <c r="J104" s="2">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4848,7 +4874,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="1">
+      <c r="J105" s="2">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4883,7 +4909,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="1">
+      <c r="J106" s="2">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4918,7 +4944,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="1">
+      <c r="J107" s="2">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4953,7 +4979,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="1">
+      <c r="J108" s="2">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -4988,7 +5014,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="1">
+      <c r="J109" s="2">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5023,7 +5049,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="1">
+      <c r="J110" s="2">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5058,7 +5084,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="1">
+      <c r="J111" s="2">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5093,7 +5119,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="1">
+      <c r="J112" s="2">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5128,7 +5154,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="1">
+      <c r="J113" s="2">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5163,7 +5189,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="1">
+      <c r="J114" s="2">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5198,7 +5224,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="1">
+      <c r="J115" s="2">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5233,7 +5259,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="1">
+      <c r="J116" s="2">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5268,7 +5294,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="1">
+      <c r="J117" s="2">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5303,7 +5329,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="1">
+      <c r="J118" s="2">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5338,7 +5364,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="1">
+      <c r="J119" s="2">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5373,7 +5399,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="1">
+      <c r="J120" s="2">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5408,7 +5434,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="1">
+      <c r="J121" s="2">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5443,7 +5469,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="1">
+      <c r="J122" s="2">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5478,7 +5504,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="1">
+      <c r="J123" s="2">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5513,7 +5539,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="1">
+      <c r="J124" s="2">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5548,7 +5574,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="1">
+      <c r="J125" s="2">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5583,7 +5609,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="1">
+      <c r="J126" s="2">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5618,7 +5644,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="1">
+      <c r="J127" s="2">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5653,7 +5679,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="1">
+      <c r="J128" s="2">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5688,7 +5714,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="1">
+      <c r="J129" s="2">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5723,7 +5749,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="1">
+      <c r="J130" s="2">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5758,7 +5784,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="1">
+      <c r="J131" s="2">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5793,7 +5819,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="1">
+      <c r="J132" s="2">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5828,7 +5854,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="1">
+      <c r="J133" s="2">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5863,7 +5889,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="1">
+      <c r="J134" s="2">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5898,7 +5924,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="1">
+      <c r="J135" s="2">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5933,7 +5959,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="1">
+      <c r="J136" s="2">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5968,7 +5994,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="1">
+      <c r="J137" s="2">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6000,7 +6026,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="1">
+      <c r="J138" s="2">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6032,7 +6058,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="1">
+      <c r="J139" s="2">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6064,7 +6090,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="1">
+      <c r="J140" s="2">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6096,7 +6122,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="1">
+      <c r="J141" s="2">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6128,7 +6154,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="1">
+      <c r="J142" s="2">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6160,7 +6186,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="1">
+      <c r="J143" s="2">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6192,7 +6218,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="1">
+      <c r="J144" s="2">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6224,7 +6250,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="1">
+      <c r="J145" s="2">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6256,7 +6282,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="1">
+      <c r="J146" s="2">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6288,7 +6314,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="1">
+      <c r="J147" s="2">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6320,7 +6346,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="1">
+      <c r="J148" s="2">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6352,7 +6378,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="1">
+      <c r="J149" s="2">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6384,7 +6410,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="1">
+      <c r="J150" s="2">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6416,7 +6442,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="1">
+      <c r="J151" s="2">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6448,7 +6474,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="1">
+      <c r="J152" s="2">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6480,7 +6506,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="1">
+      <c r="J153" s="2">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6512,7 +6538,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="1">
+      <c r="J154" s="2">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6544,7 +6570,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="1">
+      <c r="J155" s="2">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6576,7 +6602,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="1">
+      <c r="J156" s="2">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6608,7 +6634,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="1">
+      <c r="J157" s="2">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6640,7 +6666,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="1">
+      <c r="J158" s="2">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6672,7 +6698,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="1">
+      <c r="J159" s="2">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6704,7 +6730,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="1">
+      <c r="J160" s="2">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6736,7 +6762,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="1">
+      <c r="J161" s="2">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6768,7 +6794,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="1">
+      <c r="J162" s="2">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6800,7 +6826,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="1">
+      <c r="J163" s="2">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6832,7 +6858,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="1">
+      <c r="J164" s="2">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6864,7 +6890,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="1">
+      <c r="J165" s="2">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6896,7 +6922,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="1">
+      <c r="J166" s="2">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6928,7 +6954,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="1">
+      <c r="J167" s="2">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6960,7 +6986,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="1">
+      <c r="J168" s="2">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -6992,7 +7018,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="1">
+      <c r="J169" s="2">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7024,7 +7050,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="1">
+      <c r="J170" s="2">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7056,7 +7082,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="1">
+      <c r="J171" s="2">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7088,7 +7114,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="1">
+      <c r="J172" s="2">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7120,7 +7146,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="1">
+      <c r="J173" s="2">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7152,7 +7178,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="1">
+      <c r="J174" s="2">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7184,7 +7210,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="1">
+      <c r="J175" s="2">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7216,7 +7242,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="1">
+      <c r="J176" s="2">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7248,7 +7274,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="1">
+      <c r="J177" s="2">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7280,7 +7306,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="1">
+      <c r="J178" s="2">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7312,7 +7338,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="1">
+      <c r="J179" s="2">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7344,7 +7370,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="1">
+      <c r="J180" s="2">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7376,7 +7402,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="1">
+      <c r="J181" s="2">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7408,7 +7434,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="1">
+      <c r="J182" s="2">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7440,7 +7466,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="1">
+      <c r="J183" s="2">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7472,7 +7498,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="1">
+      <c r="J184" s="2">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>

<commit_message>
Atualização automática: vencimentos_tmot (26/10/2026 14:17)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_tratada.xlsx
@@ -1040,16 +1040,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1065,7 +1057,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1073,30 +1065,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1396,37 +1370,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1455,7 +1429,7 @@
       <c r="H2">
         <v>-2354.2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>40669</v>
       </c>
       <c r="K2" t="b">
@@ -1487,7 +1461,7 @@
       <c r="H3">
         <v>-934.3</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>40669</v>
       </c>
       <c r="K3" t="b">
@@ -1519,7 +1493,7 @@
       <c r="H4">
         <v>-891.7</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>44884</v>
       </c>
       <c r="K4" t="b">
@@ -1551,7 +1525,7 @@
       <c r="H5">
         <v>-589.5</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>43855</v>
       </c>
       <c r="K5" t="b">
@@ -1583,7 +1557,7 @@
       <c r="H6">
         <v>-562</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>45804</v>
       </c>
       <c r="K6" t="b">
@@ -1615,7 +1589,7 @@
       <c r="H7">
         <v>-560.5</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>45804</v>
       </c>
       <c r="K7" t="b">
@@ -1647,7 +1621,7 @@
       <c r="H8">
         <v>-531.8</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46014</v>
       </c>
       <c r="K8" t="b">
@@ -1679,7 +1653,7 @@
       <c r="H9">
         <v>-529.1</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46014</v>
       </c>
       <c r="K9" t="b">
@@ -1711,7 +1685,7 @@
       <c r="H10">
         <v>-391.8</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>32786</v>
       </c>
       <c r="K10" t="b">
@@ -1743,7 +1717,7 @@
       <c r="H11">
         <v>-391.8</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>42769</v>
       </c>
       <c r="K11" t="b">
@@ -1775,7 +1749,7 @@
       <c r="H12">
         <v>-288.8</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>34700</v>
       </c>
       <c r="K12" t="b">
@@ -1807,7 +1781,7 @@
       <c r="H13">
         <v>-206</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>41204</v>
       </c>
       <c r="K13" t="b">
@@ -1839,7 +1813,7 @@
       <c r="H14">
         <v>-186.8</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46111</v>
       </c>
       <c r="K14" t="b">
@@ -1871,7 +1845,7 @@
       <c r="H15">
         <v>-186.8</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46111</v>
       </c>
       <c r="K15" t="b">
@@ -1903,7 +1877,7 @@
       <c r="H16">
         <v>-186.8</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46111</v>
       </c>
       <c r="K16" t="b">
@@ -1935,7 +1909,7 @@
       <c r="H17">
         <v>-186.8</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46111</v>
       </c>
       <c r="K17" t="b">
@@ -1967,7 +1941,7 @@
       <c r="H18">
         <v>-186.8</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46111</v>
       </c>
       <c r="K18" t="b">
@@ -1999,7 +1973,7 @@
       <c r="H19">
         <v>-128.6</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46161</v>
       </c>
       <c r="K19" t="b">
@@ -2031,7 +2005,7 @@
       <c r="H20">
         <v>-108.2</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46242</v>
       </c>
       <c r="K20" t="b">
@@ -2063,7 +2037,7 @@
       <c r="H21">
         <v>-107</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>40979</v>
       </c>
       <c r="K21" t="b">
@@ -2095,7 +2069,7 @@
       <c r="H22">
         <v>-99.8</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46255</v>
       </c>
       <c r="K22" t="b">
@@ -2127,7 +2101,7 @@
       <c r="H23">
         <v>-54.8</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46285</v>
       </c>
       <c r="K23" t="b">
@@ -2159,7 +2133,7 @@
       <c r="H24">
         <v>-29.7</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46269</v>
       </c>
       <c r="K24" t="b">
@@ -2191,7 +2165,7 @@
       <c r="H25">
         <v>-25.6</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46282</v>
       </c>
       <c r="K25" t="b">
@@ -2223,7 +2197,7 @@
       <c r="H26">
         <v>-13.8</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46236</v>
       </c>
       <c r="K26" t="b">
@@ -2255,7 +2229,7 @@
       <c r="H27">
         <v>9.9</v>
       </c>
-      <c r="J27" s="2">
+      <c r="J27" s="1">
         <v>46354</v>
       </c>
       <c r="K27" t="b">
@@ -2287,7 +2261,7 @@
       <c r="H28">
         <v>16.2</v>
       </c>
-      <c r="J28" s="2">
+      <c r="J28" s="1">
         <v>46326</v>
       </c>
       <c r="K28" t="b">
@@ -2319,7 +2293,7 @@
       <c r="H29">
         <v>30.4</v>
       </c>
-      <c r="J29" s="2">
+      <c r="J29" s="1">
         <v>46335</v>
       </c>
       <c r="K29" t="b">
@@ -2351,7 +2325,7 @@
       <c r="H30">
         <v>33.6</v>
       </c>
-      <c r="J30" s="2">
+      <c r="J30" s="1">
         <v>46326</v>
       </c>
       <c r="K30" t="b">
@@ -2383,7 +2357,7 @@
       <c r="H31">
         <v>36.7</v>
       </c>
-      <c r="J31" s="2">
+      <c r="J31" s="1">
         <v>46326</v>
       </c>
       <c r="K31" t="b">
@@ -2415,7 +2389,7 @@
       <c r="H32">
         <v>41.4</v>
       </c>
-      <c r="J32" s="2">
+      <c r="J32" s="1">
         <v>46335</v>
       </c>
       <c r="K32" t="b">
@@ -2447,7 +2421,7 @@
       <c r="H33">
         <v>42.8</v>
       </c>
-      <c r="J33" s="2">
+      <c r="J33" s="1">
         <v>46389</v>
       </c>
       <c r="K33" t="b">
@@ -2479,7 +2453,7 @@
       <c r="H34">
         <v>45.6</v>
       </c>
-      <c r="J34" s="2">
+      <c r="J34" s="1">
         <v>46475</v>
       </c>
       <c r="K34" t="b">
@@ -2511,7 +2485,7 @@
       <c r="H35">
         <v>47.2</v>
       </c>
-      <c r="J35" s="2">
+      <c r="J35" s="1">
         <v>46391</v>
       </c>
       <c r="K35" t="b">
@@ -2543,7 +2517,7 @@
       <c r="H36">
         <v>59.1</v>
       </c>
-      <c r="J36" s="2">
+      <c r="J36" s="1">
         <v>46509</v>
       </c>
       <c r="K36" t="b">
@@ -2575,7 +2549,7 @@
       <c r="H37">
         <v>61.1</v>
       </c>
-      <c r="J37" s="2">
+      <c r="J37" s="1">
         <v>46514</v>
       </c>
       <c r="K37" t="b">
@@ -2607,7 +2581,7 @@
       <c r="H38">
         <v>67</v>
       </c>
-      <c r="J38" s="2">
+      <c r="J38" s="1">
         <v>46336</v>
       </c>
       <c r="K38" t="b">
@@ -2639,7 +2613,7 @@
       <c r="H39">
         <v>72.5</v>
       </c>
-      <c r="J39" s="2">
+      <c r="J39" s="1">
         <v>46343</v>
       </c>
       <c r="K39" t="b">
@@ -2671,7 +2645,7 @@
       <c r="H40">
         <v>74.09999999999999</v>
       </c>
-      <c r="J40" s="2">
+      <c r="J40" s="1">
         <v>46326</v>
       </c>
       <c r="K40" t="b">
@@ -2703,7 +2677,7 @@
       <c r="H41">
         <v>74.09999999999999</v>
       </c>
-      <c r="J41" s="2">
+      <c r="J41" s="1">
         <v>46326</v>
       </c>
       <c r="K41" t="b">
@@ -2735,7 +2709,7 @@
       <c r="H42">
         <v>77.5</v>
       </c>
-      <c r="J42" s="2">
+      <c r="J42" s="1">
         <v>46346</v>
       </c>
       <c r="K42" t="b">
@@ -2767,7 +2741,7 @@
       <c r="H43">
         <v>95.2</v>
       </c>
-      <c r="J43" s="2">
+      <c r="J43" s="1">
         <v>46392</v>
       </c>
       <c r="K43" t="b">
@@ -2799,7 +2773,7 @@
       <c r="H44">
         <v>100</v>
       </c>
-      <c r="J44" s="2">
+      <c r="J44" s="1">
         <v>46375</v>
       </c>
       <c r="K44" t="b">
@@ -2831,7 +2805,7 @@
       <c r="H45">
         <v>100</v>
       </c>
-      <c r="J45" s="2">
+      <c r="J45" s="1">
         <v>46375</v>
       </c>
       <c r="K45" t="b">
@@ -2863,7 +2837,7 @@
       <c r="H46">
         <v>100.3</v>
       </c>
-      <c r="J46" s="2">
+      <c r="J46" s="1">
         <v>46345</v>
       </c>
       <c r="K46" t="b">
@@ -2895,7 +2869,7 @@
       <c r="H47">
         <v>104.1</v>
       </c>
-      <c r="J47" s="2">
+      <c r="J47" s="1">
         <v>46418</v>
       </c>
       <c r="K47" t="b">
@@ -2927,7 +2901,7 @@
       <c r="H48">
         <v>106.4</v>
       </c>
-      <c r="J48" s="2">
+      <c r="J48" s="1">
         <v>46347</v>
       </c>
       <c r="K48" t="b">
@@ -2959,7 +2933,7 @@
       <c r="H49">
         <v>114.3</v>
       </c>
-      <c r="J49" s="2">
+      <c r="J49" s="1">
         <v>46418</v>
       </c>
       <c r="K49" t="b">
@@ -2991,7 +2965,7 @@
       <c r="H50">
         <v>114.8</v>
       </c>
-      <c r="J50" s="2">
+      <c r="J50" s="1">
         <v>46400</v>
       </c>
       <c r="K50" t="b">
@@ -3023,7 +2997,7 @@
       <c r="H51">
         <v>133.6</v>
       </c>
-      <c r="J51" s="2">
+      <c r="J51" s="1">
         <v>46424</v>
       </c>
       <c r="K51" t="b">
@@ -3055,7 +3029,7 @@
       <c r="H52">
         <v>135.2</v>
       </c>
-      <c r="J52" s="2">
+      <c r="J52" s="1">
         <v>46384</v>
       </c>
       <c r="K52" t="b">
@@ -3087,7 +3061,7 @@
       <c r="H53">
         <v>141.4</v>
       </c>
-      <c r="J53" s="2">
+      <c r="J53" s="1">
         <v>46395</v>
       </c>
       <c r="K53" t="b">
@@ -3119,7 +3093,7 @@
       <c r="H54">
         <v>144.2</v>
       </c>
-      <c r="J54" s="2">
+      <c r="J54" s="1">
         <v>46388</v>
       </c>
       <c r="K54" t="b">
@@ -3151,7 +3125,7 @@
       <c r="H55">
         <v>160.3</v>
       </c>
-      <c r="J55" s="2">
+      <c r="J55" s="1">
         <v>46433</v>
       </c>
       <c r="K55" t="b">
@@ -3183,7 +3157,7 @@
       <c r="H56">
         <v>177</v>
       </c>
-      <c r="J56" s="2">
+      <c r="J56" s="1">
         <v>46397</v>
       </c>
       <c r="K56" t="b">
@@ -3215,7 +3189,7 @@
       <c r="H57">
         <v>177.2</v>
       </c>
-      <c r="J57" s="2">
+      <c r="J57" s="1">
         <v>46423</v>
       </c>
       <c r="K57" t="b">
@@ -3247,7 +3221,7 @@
       <c r="H58">
         <v>177.4</v>
       </c>
-      <c r="J58" s="2">
+      <c r="J58" s="1">
         <v>46490</v>
       </c>
       <c r="K58" t="b">
@@ -3279,7 +3253,7 @@
       <c r="H59">
         <v>178.8</v>
       </c>
-      <c r="J59" s="2">
+      <c r="J59" s="1">
         <v>46384</v>
       </c>
       <c r="K59" t="b">
@@ -3311,7 +3285,7 @@
       <c r="H60">
         <v>196.2</v>
       </c>
-      <c r="J60" s="2">
+      <c r="J60" s="1">
         <v>46392</v>
       </c>
       <c r="K60" t="b">
@@ -3343,7 +3317,7 @@
       <c r="H61">
         <v>202.9</v>
       </c>
-      <c r="J61" s="2">
+      <c r="J61" s="1">
         <v>46394</v>
       </c>
       <c r="K61" t="b">
@@ -3375,7 +3349,7 @@
       <c r="H62">
         <v>211.2</v>
       </c>
-      <c r="J62" s="2">
+      <c r="J62" s="1">
         <v>46451</v>
       </c>
       <c r="K62" t="b">
@@ -3407,7 +3381,7 @@
       <c r="H63">
         <v>275.6</v>
       </c>
-      <c r="J63" s="2">
+      <c r="J63" s="1">
         <v>46459</v>
       </c>
       <c r="K63" t="b">
@@ -3439,7 +3413,7 @@
       <c r="H64">
         <v>293.4</v>
       </c>
-      <c r="J64" s="2">
+      <c r="J64" s="1">
         <v>46473</v>
       </c>
       <c r="K64" t="b">
@@ -3474,7 +3448,7 @@
       <c r="I65" t="s">
         <v>312</v>
       </c>
-      <c r="J65" s="2">
+      <c r="J65" s="1">
         <v>36557</v>
       </c>
       <c r="K65" t="b">
@@ -3509,7 +3483,7 @@
       <c r="I66" t="s">
         <v>313</v>
       </c>
-      <c r="J66" s="2">
+      <c r="J66" s="1">
         <v>38353</v>
       </c>
       <c r="K66" t="b">
@@ -3544,7 +3518,7 @@
       <c r="I67" t="s">
         <v>314</v>
       </c>
-      <c r="J67" s="2">
+      <c r="J67" s="1">
         <v>45380</v>
       </c>
       <c r="K67" t="b">
@@ -3579,7 +3553,7 @@
       <c r="I68" t="s">
         <v>315</v>
       </c>
-      <c r="J68" s="2">
+      <c r="J68" s="1">
         <v>45421</v>
       </c>
       <c r="K68" t="b">
@@ -3614,7 +3588,7 @@
       <c r="I69" t="s">
         <v>315</v>
       </c>
-      <c r="J69" s="2">
+      <c r="J69" s="1">
         <v>45428</v>
       </c>
       <c r="K69" t="b">
@@ -3649,7 +3623,7 @@
       <c r="I70" t="s">
         <v>316</v>
       </c>
-      <c r="J70" s="2">
+      <c r="J70" s="1">
         <v>45490</v>
       </c>
       <c r="K70" t="b">
@@ -3684,7 +3658,7 @@
       <c r="I71" t="s">
         <v>317</v>
       </c>
-      <c r="J71" s="2">
+      <c r="J71" s="1">
         <v>45566</v>
       </c>
       <c r="K71" t="b">
@@ -3719,7 +3693,7 @@
       <c r="I72" t="s">
         <v>318</v>
       </c>
-      <c r="J72" s="2">
+      <c r="J72" s="1">
         <v>45986</v>
       </c>
       <c r="K72" t="b">
@@ -3754,7 +3728,7 @@
       <c r="I73" t="s">
         <v>319</v>
       </c>
-      <c r="J73" s="2">
+      <c r="J73" s="1">
         <v>46197</v>
       </c>
       <c r="K73" t="b">
@@ -3789,7 +3763,7 @@
       <c r="I74" t="s">
         <v>320</v>
       </c>
-      <c r="J74" s="2">
+      <c r="J74" s="1">
         <v>46212</v>
       </c>
       <c r="K74" t="b">
@@ -3824,7 +3798,7 @@
       <c r="I75" t="s">
         <v>320</v>
       </c>
-      <c r="J75" s="2">
+      <c r="J75" s="1">
         <v>46225</v>
       </c>
       <c r="K75" t="b">
@@ -3859,7 +3833,7 @@
       <c r="I76" t="s">
         <v>320</v>
       </c>
-      <c r="J76" s="2">
+      <c r="J76" s="1">
         <v>46235</v>
       </c>
       <c r="K76" t="b">
@@ -3894,7 +3868,7 @@
       <c r="I77" t="s">
         <v>321</v>
       </c>
-      <c r="J77" s="2">
+      <c r="J77" s="1">
         <v>46345</v>
       </c>
       <c r="K77" t="b">
@@ -3929,7 +3903,7 @@
       <c r="I78" t="s">
         <v>321</v>
       </c>
-      <c r="J78" s="2">
+      <c r="J78" s="1">
         <v>46360</v>
       </c>
       <c r="K78" t="b">
@@ -3964,7 +3938,7 @@
       <c r="I79" t="s">
         <v>322</v>
       </c>
-      <c r="J79" s="2">
+      <c r="J79" s="1">
         <v>46367</v>
       </c>
       <c r="K79" t="b">
@@ -3999,7 +3973,7 @@
       <c r="I80" t="s">
         <v>322</v>
       </c>
-      <c r="J80" s="2">
+      <c r="J80" s="1">
         <v>46368</v>
       </c>
       <c r="K80" t="b">
@@ -4034,7 +4008,7 @@
       <c r="I81" t="s">
         <v>322</v>
       </c>
-      <c r="J81" s="2">
+      <c r="J81" s="1">
         <v>46375</v>
       </c>
       <c r="K81" t="b">
@@ -4069,7 +4043,7 @@
       <c r="I82" t="s">
         <v>322</v>
       </c>
-      <c r="J82" s="2">
+      <c r="J82" s="1">
         <v>46387</v>
       </c>
       <c r="K82" t="b">
@@ -4104,7 +4078,7 @@
       <c r="I83" t="s">
         <v>322</v>
       </c>
-      <c r="J83" s="2">
+      <c r="J83" s="1">
         <v>46387</v>
       </c>
       <c r="K83" t="b">
@@ -4139,7 +4113,7 @@
       <c r="I84" t="s">
         <v>322</v>
       </c>
-      <c r="J84" s="2">
+      <c r="J84" s="1">
         <v>46387</v>
       </c>
       <c r="K84" t="b">
@@ -4174,7 +4148,7 @@
       <c r="I85" t="s">
         <v>322</v>
       </c>
-      <c r="J85" s="2">
+      <c r="J85" s="1">
         <v>46388</v>
       </c>
       <c r="K85" t="b">
@@ -4209,7 +4183,7 @@
       <c r="I86" t="s">
         <v>323</v>
       </c>
-      <c r="J86" s="2">
+      <c r="J86" s="1">
         <v>46401</v>
       </c>
       <c r="K86" t="b">
@@ -4244,7 +4218,7 @@
       <c r="I87" t="s">
         <v>323</v>
       </c>
-      <c r="J87" s="2">
+      <c r="J87" s="1">
         <v>46401</v>
       </c>
       <c r="K87" t="b">
@@ -4279,7 +4253,7 @@
       <c r="I88" t="s">
         <v>323</v>
       </c>
-      <c r="J88" s="2">
+      <c r="J88" s="1">
         <v>46401</v>
       </c>
       <c r="K88" t="b">
@@ -4314,7 +4288,7 @@
       <c r="I89" t="s">
         <v>323</v>
       </c>
-      <c r="J89" s="2">
+      <c r="J89" s="1">
         <v>46403</v>
       </c>
       <c r="K89" t="b">
@@ -4349,7 +4323,7 @@
       <c r="I90" t="s">
         <v>323</v>
       </c>
-      <c r="J90" s="2">
+      <c r="J90" s="1">
         <v>46412</v>
       </c>
       <c r="K90" t="b">
@@ -4384,7 +4358,7 @@
       <c r="I91" t="s">
         <v>323</v>
       </c>
-      <c r="J91" s="2">
+      <c r="J91" s="1">
         <v>46412</v>
       </c>
       <c r="K91" t="b">
@@ -4419,7 +4393,7 @@
       <c r="I92" t="s">
         <v>323</v>
       </c>
-      <c r="J92" s="2">
+      <c r="J92" s="1">
         <v>46424</v>
       </c>
       <c r="K92" t="b">
@@ -4454,7 +4428,7 @@
       <c r="I93" t="s">
         <v>324</v>
       </c>
-      <c r="J93" s="2">
+      <c r="J93" s="1">
         <v>46427</v>
       </c>
       <c r="K93" t="b">
@@ -4489,7 +4463,7 @@
       <c r="I94" t="s">
         <v>324</v>
       </c>
-      <c r="J94" s="2">
+      <c r="J94" s="1">
         <v>46427</v>
       </c>
       <c r="K94" t="b">
@@ -4524,7 +4498,7 @@
       <c r="I95" t="s">
         <v>324</v>
       </c>
-      <c r="J95" s="2">
+      <c r="J95" s="1">
         <v>46437</v>
       </c>
       <c r="K95" t="b">
@@ -4559,7 +4533,7 @@
       <c r="I96" t="s">
         <v>324</v>
       </c>
-      <c r="J96" s="2">
+      <c r="J96" s="1">
         <v>46451</v>
       </c>
       <c r="K96" t="b">
@@ -4594,7 +4568,7 @@
       <c r="I97" t="s">
         <v>324</v>
       </c>
-      <c r="J97" s="2">
+      <c r="J97" s="1">
         <v>46451</v>
       </c>
       <c r="K97" t="b">
@@ -4629,7 +4603,7 @@
       <c r="I98" t="s">
         <v>325</v>
       </c>
-      <c r="J98" s="2">
+      <c r="J98" s="1">
         <v>46455</v>
       </c>
       <c r="K98" t="b">
@@ -4664,7 +4638,7 @@
       <c r="I99" t="s">
         <v>325</v>
       </c>
-      <c r="J99" s="2">
+      <c r="J99" s="1">
         <v>46456</v>
       </c>
       <c r="K99" t="b">
@@ -4699,7 +4673,7 @@
       <c r="I100" t="s">
         <v>325</v>
       </c>
-      <c r="J100" s="2">
+      <c r="J100" s="1">
         <v>46457</v>
       </c>
       <c r="K100" t="b">
@@ -4734,7 +4708,7 @@
       <c r="I101" t="s">
         <v>325</v>
       </c>
-      <c r="J101" s="2">
+      <c r="J101" s="1">
         <v>46462</v>
       </c>
       <c r="K101" t="b">
@@ -4769,7 +4743,7 @@
       <c r="I102" t="s">
         <v>325</v>
       </c>
-      <c r="J102" s="2">
+      <c r="J102" s="1">
         <v>46464</v>
       </c>
       <c r="K102" t="b">
@@ -4804,7 +4778,7 @@
       <c r="I103" t="s">
         <v>325</v>
       </c>
-      <c r="J103" s="2">
+      <c r="J103" s="1">
         <v>46470</v>
       </c>
       <c r="K103" t="b">
@@ -4839,7 +4813,7 @@
       <c r="I104" t="s">
         <v>325</v>
       </c>
-      <c r="J104" s="2">
+      <c r="J104" s="1">
         <v>46485</v>
       </c>
       <c r="K104" t="b">
@@ -4874,7 +4848,7 @@
       <c r="I105" t="s">
         <v>326</v>
       </c>
-      <c r="J105" s="2">
+      <c r="J105" s="1">
         <v>46499</v>
       </c>
       <c r="K105" t="b">
@@ -4909,7 +4883,7 @@
       <c r="I106" t="s">
         <v>326</v>
       </c>
-      <c r="J106" s="2">
+      <c r="J106" s="1">
         <v>46504</v>
       </c>
       <c r="K106" t="b">
@@ -4944,7 +4918,7 @@
       <c r="I107" t="s">
         <v>326</v>
       </c>
-      <c r="J107" s="2">
+      <c r="J107" s="1">
         <v>46507</v>
       </c>
       <c r="K107" t="b">
@@ -4979,7 +4953,7 @@
       <c r="I108" t="s">
         <v>326</v>
       </c>
-      <c r="J108" s="2">
+      <c r="J108" s="1">
         <v>46508</v>
       </c>
       <c r="K108" t="b">
@@ -5014,7 +4988,7 @@
       <c r="I109" t="s">
         <v>326</v>
       </c>
-      <c r="J109" s="2">
+      <c r="J109" s="1">
         <v>46512</v>
       </c>
       <c r="K109" t="b">
@@ -5049,7 +5023,7 @@
       <c r="I110" t="s">
         <v>327</v>
       </c>
-      <c r="J110" s="2">
+      <c r="J110" s="1">
         <v>46528</v>
       </c>
       <c r="K110" t="b">
@@ -5084,7 +5058,7 @@
       <c r="I111" t="s">
         <v>327</v>
       </c>
-      <c r="J111" s="2">
+      <c r="J111" s="1">
         <v>46529</v>
       </c>
       <c r="K111" t="b">
@@ -5119,7 +5093,7 @@
       <c r="I112" t="s">
         <v>327</v>
       </c>
-      <c r="J112" s="2">
+      <c r="J112" s="1">
         <v>46537</v>
       </c>
       <c r="K112" t="b">
@@ -5154,7 +5128,7 @@
       <c r="I113" t="s">
         <v>328</v>
       </c>
-      <c r="J113" s="2">
+      <c r="J113" s="1">
         <v>46546</v>
       </c>
       <c r="K113" t="b">
@@ -5189,7 +5163,7 @@
       <c r="I114" t="s">
         <v>328</v>
       </c>
-      <c r="J114" s="2">
+      <c r="J114" s="1">
         <v>46547</v>
       </c>
       <c r="K114" t="b">
@@ -5224,7 +5198,7 @@
       <c r="I115" t="s">
         <v>328</v>
       </c>
-      <c r="J115" s="2">
+      <c r="J115" s="1">
         <v>46547</v>
       </c>
       <c r="K115" t="b">
@@ -5259,7 +5233,7 @@
       <c r="I116" t="s">
         <v>328</v>
       </c>
-      <c r="J116" s="2">
+      <c r="J116" s="1">
         <v>46551</v>
       </c>
       <c r="K116" t="b">
@@ -5294,7 +5268,7 @@
       <c r="I117" t="s">
         <v>328</v>
       </c>
-      <c r="J117" s="2">
+      <c r="J117" s="1">
         <v>46560</v>
       </c>
       <c r="K117" t="b">
@@ -5329,7 +5303,7 @@
       <c r="I118" t="s">
         <v>328</v>
       </c>
-      <c r="J118" s="2">
+      <c r="J118" s="1">
         <v>46568</v>
       </c>
       <c r="K118" t="b">
@@ -5364,7 +5338,7 @@
       <c r="I119" t="s">
         <v>329</v>
       </c>
-      <c r="J119" s="2">
+      <c r="J119" s="1">
         <v>46592</v>
       </c>
       <c r="K119" t="b">
@@ -5399,7 +5373,7 @@
       <c r="I120" t="s">
         <v>329</v>
       </c>
-      <c r="J120" s="2">
+      <c r="J120" s="1">
         <v>46603</v>
       </c>
       <c r="K120" t="b">
@@ -5434,7 +5408,7 @@
       <c r="I121" t="s">
         <v>330</v>
       </c>
-      <c r="J121" s="2">
+      <c r="J121" s="1">
         <v>46611</v>
       </c>
       <c r="K121" t="b">
@@ -5469,7 +5443,7 @@
       <c r="I122" t="s">
         <v>330</v>
       </c>
-      <c r="J122" s="2">
+      <c r="J122" s="1">
         <v>46631</v>
       </c>
       <c r="K122" t="b">
@@ -5504,7 +5478,7 @@
       <c r="I123" t="s">
         <v>331</v>
       </c>
-      <c r="J123" s="2">
+      <c r="J123" s="1">
         <v>46645</v>
       </c>
       <c r="K123" t="b">
@@ -5539,7 +5513,7 @@
       <c r="I124" t="s">
         <v>331</v>
       </c>
-      <c r="J124" s="2">
+      <c r="J124" s="1">
         <v>46646</v>
       </c>
       <c r="K124" t="b">
@@ -5574,7 +5548,7 @@
       <c r="I125" t="s">
         <v>331</v>
       </c>
-      <c r="J125" s="2">
+      <c r="J125" s="1">
         <v>46652</v>
       </c>
       <c r="K125" t="b">
@@ -5609,7 +5583,7 @@
       <c r="I126" t="s">
         <v>331</v>
       </c>
-      <c r="J126" s="2">
+      <c r="J126" s="1">
         <v>46658</v>
       </c>
       <c r="K126" t="b">
@@ -5644,7 +5618,7 @@
       <c r="I127" t="s">
         <v>331</v>
       </c>
-      <c r="J127" s="2">
+      <c r="J127" s="1">
         <v>46659</v>
       </c>
       <c r="K127" t="b">
@@ -5679,7 +5653,7 @@
       <c r="I128" t="s">
         <v>332</v>
       </c>
-      <c r="J128" s="2">
+      <c r="J128" s="1">
         <v>46254</v>
       </c>
       <c r="K128" t="b">
@@ -5714,7 +5688,7 @@
       <c r="I129" t="s">
         <v>333</v>
       </c>
-      <c r="J129" s="2">
+      <c r="J129" s="1">
         <v>46293</v>
       </c>
       <c r="K129" t="b">
@@ -5749,7 +5723,7 @@
       <c r="I130" t="s">
         <v>333</v>
       </c>
-      <c r="J130" s="2">
+      <c r="J130" s="1">
         <v>46296</v>
       </c>
       <c r="K130" t="b">
@@ -5784,7 +5758,7 @@
       <c r="I131" t="s">
         <v>334</v>
       </c>
-      <c r="J131" s="2">
+      <c r="J131" s="1">
         <v>46305</v>
       </c>
       <c r="K131" t="b">
@@ -5819,7 +5793,7 @@
       <c r="I132" t="s">
         <v>335</v>
       </c>
-      <c r="J132" s="2">
+      <c r="J132" s="1">
         <v>46317</v>
       </c>
       <c r="K132" t="b">
@@ -5854,7 +5828,7 @@
       <c r="I133" t="s">
         <v>321</v>
       </c>
-      <c r="J133" s="2">
+      <c r="J133" s="1">
         <v>46333</v>
       </c>
       <c r="K133" t="b">
@@ -5889,7 +5863,7 @@
       <c r="I134" t="s">
         <v>336</v>
       </c>
-      <c r="J134" s="2">
+      <c r="J134" s="1">
         <v>46338</v>
       </c>
       <c r="K134" t="b">
@@ -5924,7 +5898,7 @@
       <c r="I135" t="s">
         <v>336</v>
       </c>
-      <c r="J135" s="2">
+      <c r="J135" s="1">
         <v>46338</v>
       </c>
       <c r="K135" t="b">
@@ -5959,7 +5933,7 @@
       <c r="I136" t="s">
         <v>337</v>
       </c>
-      <c r="J136" s="2">
+      <c r="J136" s="1">
         <v>46341</v>
       </c>
       <c r="K136" t="b">
@@ -5994,7 +5968,7 @@
       <c r="I137" t="s">
         <v>338</v>
       </c>
-      <c r="J137" s="2">
+      <c r="J137" s="1">
         <v>46344</v>
       </c>
       <c r="K137" t="b">
@@ -6026,7 +6000,7 @@
       <c r="H138">
         <v>-1476</v>
       </c>
-      <c r="J138" s="2">
+      <c r="J138" s="1">
         <v>43773</v>
       </c>
       <c r="K138" t="b">
@@ -6058,7 +6032,7 @@
       <c r="H139">
         <v>-1469</v>
       </c>
-      <c r="J139" s="2">
+      <c r="J139" s="1">
         <v>43773</v>
       </c>
       <c r="K139" t="b">
@@ -6090,7 +6064,7 @@
       <c r="H140">
         <v>-1280</v>
       </c>
-      <c r="J140" s="2">
+      <c r="J140" s="1">
         <v>45295</v>
       </c>
       <c r="K140" t="b">
@@ -6122,7 +6096,7 @@
       <c r="H141">
         <v>-1141</v>
       </c>
-      <c r="J141" s="2">
+      <c r="J141" s="1">
         <v>45617</v>
       </c>
       <c r="K141" t="b">
@@ -6154,7 +6128,7 @@
       <c r="H142">
         <v>-1073</v>
       </c>
-      <c r="J142" s="2">
+      <c r="J142" s="1">
         <v>45677</v>
       </c>
       <c r="K142" t="b">
@@ -6186,7 +6160,7 @@
       <c r="H143">
         <v>-78</v>
       </c>
-      <c r="J143" s="2">
+      <c r="J143" s="1">
         <v>46254</v>
       </c>
       <c r="K143" t="b">
@@ -6218,7 +6192,7 @@
       <c r="H144">
         <v>-78</v>
       </c>
-      <c r="J144" s="2">
+      <c r="J144" s="1">
         <v>46254</v>
       </c>
       <c r="K144" t="b">
@@ -6250,7 +6224,7 @@
       <c r="H145">
         <v>-40</v>
       </c>
-      <c r="J145" s="2">
+      <c r="J145" s="1">
         <v>46092</v>
       </c>
       <c r="K145" t="b">
@@ -6282,7 +6256,7 @@
       <c r="H146">
         <v>-4</v>
       </c>
-      <c r="J146" s="2">
+      <c r="J146" s="1">
         <v>46298</v>
       </c>
       <c r="K146" t="b">
@@ -6314,7 +6288,7 @@
       <c r="H147">
         <v>43</v>
       </c>
-      <c r="J147" s="2">
+      <c r="J147" s="1">
         <v>46440</v>
       </c>
       <c r="K147" t="b">
@@ -6346,7 +6320,7 @@
       <c r="H148">
         <v>43</v>
       </c>
-      <c r="J148" s="2">
+      <c r="J148" s="1">
         <v>46440</v>
       </c>
       <c r="K148" t="b">
@@ -6378,7 +6352,7 @@
       <c r="H149">
         <v>72</v>
       </c>
-      <c r="J149" s="2">
+      <c r="J149" s="1">
         <v>46386</v>
       </c>
       <c r="K149" t="b">
@@ -6410,7 +6384,7 @@
       <c r="H150">
         <v>79</v>
       </c>
-      <c r="J150" s="2">
+      <c r="J150" s="1">
         <v>46326</v>
       </c>
       <c r="K150" t="b">
@@ -6442,7 +6416,7 @@
       <c r="H151">
         <v>79</v>
       </c>
-      <c r="J151" s="2">
+      <c r="J151" s="1">
         <v>46326</v>
       </c>
       <c r="K151" t="b">
@@ -6474,7 +6448,7 @@
       <c r="H152">
         <v>83</v>
       </c>
-      <c r="J152" s="2">
+      <c r="J152" s="1">
         <v>46395</v>
       </c>
       <c r="K152" t="b">
@@ -6506,7 +6480,7 @@
       <c r="H153">
         <v>102</v>
       </c>
-      <c r="J153" s="2">
+      <c r="J153" s="1">
         <v>46463</v>
       </c>
       <c r="K153" t="b">
@@ -6538,7 +6512,7 @@
       <c r="H154">
         <v>106</v>
       </c>
-      <c r="J154" s="2">
+      <c r="J154" s="1">
         <v>46423</v>
       </c>
       <c r="K154" t="b">
@@ -6570,7 +6544,7 @@
       <c r="H155">
         <v>107</v>
       </c>
-      <c r="J155" s="2">
+      <c r="J155" s="1">
         <v>46376</v>
       </c>
       <c r="K155" t="b">
@@ -6602,7 +6576,7 @@
       <c r="H156">
         <v>163</v>
       </c>
-      <c r="J156" s="2">
+      <c r="J156" s="1">
         <v>46592</v>
       </c>
       <c r="K156" t="b">
@@ -6634,7 +6608,7 @@
       <c r="H157">
         <v>168</v>
       </c>
-      <c r="J157" s="2">
+      <c r="J157" s="1">
         <v>46456</v>
       </c>
       <c r="K157" t="b">
@@ -6666,7 +6640,7 @@
       <c r="H158">
         <v>170</v>
       </c>
-      <c r="J158" s="2">
+      <c r="J158" s="1">
         <v>46458</v>
       </c>
       <c r="K158" t="b">
@@ -6698,7 +6672,7 @@
       <c r="H159">
         <v>188</v>
       </c>
-      <c r="J159" s="2">
+      <c r="J159" s="1">
         <v>46416</v>
       </c>
       <c r="K159" t="b">
@@ -6730,7 +6704,7 @@
       <c r="H160">
         <v>232</v>
       </c>
-      <c r="J160" s="2">
+      <c r="J160" s="1">
         <v>46509</v>
       </c>
       <c r="K160" t="b">
@@ -6762,7 +6736,7 @@
       <c r="H161">
         <v>238</v>
       </c>
-      <c r="J161" s="2">
+      <c r="J161" s="1">
         <v>46513</v>
       </c>
       <c r="K161" t="b">
@@ -6794,7 +6768,7 @@
       <c r="H162">
         <v>239</v>
       </c>
-      <c r="J162" s="2">
+      <c r="J162" s="1">
         <v>46445</v>
       </c>
       <c r="K162" t="b">
@@ -6826,7 +6800,7 @@
       <c r="H163">
         <v>239</v>
       </c>
-      <c r="J163" s="2">
+      <c r="J163" s="1">
         <v>46445</v>
       </c>
       <c r="K163" t="b">
@@ -6858,7 +6832,7 @@
       <c r="H164">
         <v>248</v>
       </c>
-      <c r="J164" s="2">
+      <c r="J164" s="1">
         <v>46592</v>
       </c>
       <c r="K164" t="b">
@@ -6890,7 +6864,7 @@
       <c r="H165">
         <v>250</v>
       </c>
-      <c r="J165" s="2">
+      <c r="J165" s="1">
         <v>46461</v>
       </c>
       <c r="K165" t="b">
@@ -6922,7 +6896,7 @@
       <c r="H166">
         <v>256</v>
       </c>
-      <c r="J166" s="2">
+      <c r="J166" s="1">
         <v>46622</v>
       </c>
       <c r="K166" t="b">
@@ -6954,7 +6928,7 @@
       <c r="H167">
         <v>331</v>
       </c>
-      <c r="J167" s="2">
+      <c r="J167" s="1">
         <v>46582</v>
       </c>
       <c r="K167" t="b">
@@ -6986,7 +6960,7 @@
       <c r="H168">
         <v>335</v>
       </c>
-      <c r="J168" s="2">
+      <c r="J168" s="1">
         <v>46513</v>
       </c>
       <c r="K168" t="b">
@@ -7018,7 +6992,7 @@
       <c r="H169">
         <v>363</v>
       </c>
-      <c r="J169" s="2">
+      <c r="J169" s="1">
         <v>46638</v>
       </c>
       <c r="K169" t="b">
@@ -7050,7 +7024,7 @@
       <c r="H170">
         <v>380</v>
       </c>
-      <c r="J170" s="2">
+      <c r="J170" s="1">
         <v>46530</v>
       </c>
       <c r="K170" t="b">
@@ -7082,7 +7056,7 @@
       <c r="H171">
         <v>403</v>
       </c>
-      <c r="J171" s="2">
+      <c r="J171" s="1">
         <v>46648</v>
       </c>
       <c r="K171" t="b">
@@ -7114,7 +7088,7 @@
       <c r="H172">
         <v>403</v>
       </c>
-      <c r="J172" s="2">
+      <c r="J172" s="1">
         <v>46648</v>
       </c>
       <c r="K172" t="b">
@@ -7146,7 +7120,7 @@
       <c r="H173">
         <v>409</v>
       </c>
-      <c r="J173" s="2">
+      <c r="J173" s="1">
         <v>46548</v>
       </c>
       <c r="K173" t="b">
@@ -7178,7 +7152,7 @@
       <c r="H174">
         <v>488</v>
       </c>
-      <c r="J174" s="2">
+      <c r="J174" s="1">
         <v>46190</v>
       </c>
       <c r="K174" t="b">
@@ -7210,7 +7184,7 @@
       <c r="H175">
         <v>533</v>
       </c>
-      <c r="J175" s="2">
+      <c r="J175" s="1">
         <v>46634</v>
       </c>
       <c r="K175" t="b">
@@ -7242,7 +7216,7 @@
       <c r="H176">
         <v>648</v>
       </c>
-      <c r="J176" s="2">
+      <c r="J176" s="1">
         <v>46377</v>
       </c>
       <c r="K176" t="b">
@@ -7274,7 +7248,7 @@
       <c r="H177">
         <v>648</v>
       </c>
-      <c r="J177" s="2">
+      <c r="J177" s="1">
         <v>46377</v>
       </c>
       <c r="K177" t="b">
@@ -7306,7 +7280,7 @@
       <c r="H178">
         <v>777</v>
       </c>
-      <c r="J178" s="2">
+      <c r="J178" s="1">
         <v>46396</v>
       </c>
       <c r="K178" t="b">
@@ -7338,7 +7312,7 @@
       <c r="H179">
         <v>777</v>
       </c>
-      <c r="J179" s="2">
+      <c r="J179" s="1">
         <v>46396</v>
       </c>
       <c r="K179" t="b">
@@ -7370,7 +7344,7 @@
       <c r="H180">
         <v>1588</v>
       </c>
-      <c r="J180" s="2">
+      <c r="J180" s="1">
         <v>46559</v>
       </c>
       <c r="K180" t="b">
@@ -7402,7 +7376,7 @@
       <c r="H181">
         <v>1588</v>
       </c>
-      <c r="J181" s="2">
+      <c r="J181" s="1">
         <v>46559</v>
       </c>
       <c r="K181" t="b">
@@ -7434,7 +7408,7 @@
       <c r="H182">
         <v>25565</v>
       </c>
-      <c r="J182" s="2">
+      <c r="J182" s="1">
         <v>46190</v>
       </c>
       <c r="K182" t="b">
@@ -7466,7 +7440,7 @@
       <c r="H183">
         <v>25567</v>
       </c>
-      <c r="J183" s="2">
+      <c r="J183" s="1">
         <v>46190</v>
       </c>
       <c r="K183" t="b">
@@ -7498,7 +7472,7 @@
       <c r="H184">
         <v>31293</v>
       </c>
-      <c r="J184" s="2">
+      <c r="J184" s="1">
         <v>46190</v>
       </c>
       <c r="K184" t="b">

</xml_diff>